<commit_message>
Rescore + rebuild downstream artifacts with partial gap-fill applied
After fill_fundamentals_gaps.py patched ~600 rows / ~2500 cells before
yfinance rate-limited, 638 yartseva_score values shifted (better
inputs flowed into the composite). Refresh the downstream:
  - asymmetry_global.csv: rebuilt from rescored per-country CSVs.
  - asymmetry_harvard_workbook.xlsx: top-50 ranking + per-name sheets.
  - top10_by_country_asymmetry.{csv,xlsx}: value+contra ranking.
  - top10_by_country_inflection.{csv,xlsx}: inflection/breakout ranking.

Top-50 verdict mix unchanged at 26 GREEN / 5 YELLOW / 0 RED /
19 UNRESEARCHED.

Bulk gap-fill on the remaining ~90 files is parked - yfinance
rate-limit is sticky in this session. Re-run when limits clear:
  python3 fill_fundamentals_gaps.py --workers 4

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/asymmetry_harvard_workbook.xlsx
+++ b/asymmetry_harvard_workbook.xlsx
@@ -905,7 +905,7 @@
     <row r="12" ht="22" customHeight="1">
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>This workbook documents the top-50 names from a global cross-listing universe of 19,750 equities ranked by an entry-today asymmetry score that blends Yartseva inflection signals, Pew sub-book / net-cash floors, Berezin growth quality, and an intrinsic-discount overlay. Each candidate has been qualitatively reviewed and assigned a verdict of Green (high-conviction), Yellow (risk-flagged), Red (avoid) or — where due diligence remains incomplete — Unresearched. Sheets are sequenced as Cover · Methodology · Index · per-name pages · Coverage · References.</t>
+          <t>This workbook documents the top-50 names from a global cross-listing universe of 19,749 equities ranked by an entry-today asymmetry score that blends Yartseva inflection signals, Pew sub-book / net-cash floors, Berezin growth quality, and an intrinsic-discount overlay. Each candidate has been qualitatively reviewed and assigned a verdict of Green (high-conviction), Yellow (risk-flagged), Red (avoid) or — where due diligence remains incomplete — Unresearched. Sheets are sequenced as Cover · Methodology · Index · per-name pages · Coverage · References.</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
     <row r="22" ht="36" customHeight="1">
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>19,750</t>
+          <t>19,749</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
@@ -26400,7 +26400,7 @@
         </is>
       </c>
       <c r="C5" s="50" t="n">
-        <v>19750</v>
+        <v>19749</v>
       </c>
       <c r="D5" s="34" t="n">
         <v>123</v>
@@ -26412,10 +26412,10 @@
         <v>130</v>
       </c>
       <c r="G5" s="34" t="n">
-        <v>19290</v>
+        <v>19289</v>
       </c>
       <c r="H5" s="51" t="n">
-        <v>2.329113924050633</v>
+        <v>2.329231859841005</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">

</xml_diff>

<commit_message>
Switch single font from Calibri to Cambria (Harvard-style serif)
User direction: Harvard aesthetic, not Calibri. Cambria is the closest
widely-available Harvard-style serif — Microsoft's bundled approximation
of Adobe Garamond / Sabon, renders cleanly in Excel on Windows / Mac /
LibreOffice. Single character of change in two files; all 5 workbooks
rebuilt and verified using Cambria 10pt exclusively.

Verification:
  Cover sheet:        {('Cambria', 10.0)}  (only one font in use)
  Per-name sheet:     {('Cambria', 10.0)}

Builders updated:
  build_harvard_workbook.py    FONT_NAME = "Cambria"
  top_n_by_country.py          FONT_NAME = 'Cambria'

Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/asymmetry_harvard_workbook.xlsx
+++ b/asymmetry_harvard_workbook.xlsx
@@ -84,42 +84,42 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Cambria"/>
       <b val="1"/>
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Cambria"/>
       <i val="1"/>
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Cambria"/>
       <i val="1"/>
       <color rgb="00707070"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Cambria"/>
       <b val="1"/>
       <color rgb="00707070"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Cambria"/>
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Cambria"/>
       <b val="1"/>
       <color rgb="00404040"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Cambria"/>
       <color rgb="00707070"/>
       <sz val="10"/>
     </font>

</xml_diff>

<commit_message>
Coverage attack: yahoo_chart + fdb sector + stooq + derive fills
- price: 91.8% -> 94.5% (Yahoo chart fill + small Stooq contribution)
- pct_off_52w_high: 0% -> 33.1% (Yahoo v8/chart endpoint)
- market_cap: 91.7% -> 94.0% (derived from price * shares_outstanding)
- sector: 88.7% -> 95.0% (FinanceDatabase hydration)
- industry: 74.4% -> 80.0% (FinanceDatabase hydration)
- country: 0% -> 98.4% (new column, FinanceDatabase)
- ev_revenue: 85.4% -> 87.4% (derive from ev_sales * revenue_ttm)
- cash_pct_mcap: 89.5% -> 91.7%, net_cash_pct_mcap 84.6% -> 86.7%

New apply scripts: apply_yahoo_chart, apply_stooq_fill, derive_missing_columns,
fdb_sector_hydrate. Rebuilt all 8 workbooks; archetypes refreshed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/asymmetry_harvard_workbook.xlsx
+++ b/asymmetry_harvard_workbook.xlsx
@@ -757,7 +757,7 @@
     <row r="11" ht="24" customHeight="1">
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>23,190</t>
+          <t>23,688</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -782,7 +782,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>22,716</t>
+          <t>23,214</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>This workbook documents the top 50 names from a global universe of 23,190 equities ranked by an entry-today asymmetry score. The upside leg weights factors Anna Yartseva (CAFE WP 33, 2025) finds predictive of 10-bagger outcomes — FCF yield, book-to-market, small size, profitability level, asset-growth gate, contra-momentum. The downside floor leg combines Graham net-net, cash &gt; EV, sub-book and negative-EV signals. Each candidate has been qualitatively reviewed and assigned a verdict of GREEN (high-conviction), YELLOW (risk-flagged), RED (avoid) or UNRESEARCHED. Sheets sequence as Cover, Methodology, Index, per-name pages, Coverage, References.</t>
+          <t>This workbook documents the top 50 names from a global universe of 23,688 equities ranked by an entry-today asymmetry score. The upside leg weights factors Anna Yartseva (CAFE WP 33, 2025) finds predictive of 10-bagger outcomes — FCF yield, book-to-market, small size, profitability level, asset-growth gate, contra-momentum. The downside floor leg combines Graham net-net, cash &gt; EV, sub-book and negative-EV signals. Each candidate has been qualitatively reviewed and assigned a verdict of GREEN (high-conviction), YELLOW (risk-flagged), RED (avoid) or UNRESEARCHED. Sheets sequence as Cover, Methodology, Index, per-name pages, Coverage, References.</t>
         </is>
       </c>
     </row>
@@ -25433,7 +25433,7 @@
         </is>
       </c>
       <c r="C5" s="42" t="n">
-        <v>23190</v>
+        <v>23688</v>
       </c>
       <c r="D5" s="28" t="n">
         <v>131</v>
@@ -25445,10 +25445,10 @@
         <v>132</v>
       </c>
       <c r="G5" s="28" t="n">
-        <v>22716</v>
+        <v>23214</v>
       </c>
       <c r="H5" s="43" t="n">
-        <v>2.043984476067271</v>
+        <v>2.001013171225937</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
@@ -25573,16 +25573,16 @@
         <v>2</v>
       </c>
       <c r="E13" s="31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" s="31" t="n">
         <v>0</v>
       </c>
       <c r="G13" s="31" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H13" s="33" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
Finish background tasks — terminal coverage state
All harvest/enrichment pipelines driven to completion:
- EDGAR: 8,021/8,021 unique CIKs, all stages done (the prior "10,433"
  was the ticker count; many tickers share a CIK). XBRL + Form 4 +
  DEF 14A caches all complete.
- yahoo_chart_fill: finished remaining 1,843 → 24,411 price rows
  (1,147 unavailable = no Yahoo chart for those symbols).
- ticker_yf: 25,451/25,558 (99.6%); the 107 stragglers genuinely
  unavailable on Yahoo quoteSummary (warm OK, every fetch returns
  empty) — terminal.

Folded all collected data into the master (apply_ticker_yf +
apply_yahoo_chart + fill_gaps + enrich + archetype_tags + enrich) and
regenerated all 8 workbooks. Verified: 0 nan/inf cells, all builders
rc=0, uniform Harvard aesthetic retained.
</commit_message>
<xml_diff>
--- a/asymmetry_harvard_workbook.xlsx
+++ b/asymmetry_harvard_workbook.xlsx
@@ -754,7 +754,7 @@
     <row r="11" ht="24" customHeight="1">
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>24,603</t>
+          <t>24,899</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>24,130</t>
+          <t>24,426</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>This workbook documents the top 50 names from a global universe of 24,603 equities ranked by an entry-today asymmetry score. The upside leg weights factors Anna Yartseva (CAFE WP 33, 2025) finds predictive of 10-bagger outcomes — FCF yield, book-to-market, small size, profitability level, asset-growth gate, contra-momentum. The downside floor leg combines Graham net-net, cash &gt; EV, sub-book and negative-EV signals. Each candidate has been qualitatively reviewed and assigned a verdict of GREEN (high-conviction), YELLOW (risk-flagged), RED (avoid) or UNRESEARCHED. Sheets sequence as Cover, Methodology, Index, per-name pages, Coverage, References.</t>
+          <t>This workbook documents the top 50 names from a global universe of 24,899 equities ranked by an entry-today asymmetry score. The upside leg weights factors Anna Yartseva (CAFE WP 33, 2025) finds predictive of 10-bagger outcomes — FCF yield, book-to-market, small size, profitability level, asset-growth gate, contra-momentum. The downside floor leg combines Graham net-net, cash &gt; EV, sub-book and negative-EV signals. Each candidate has been qualitatively reviewed and assigned a verdict of GREEN (high-conviction), YELLOW (risk-flagged), RED (avoid) or UNRESEARCHED. Sheets sequence as Cover, Methodology, Index, per-name pages, Coverage, References.</t>
         </is>
       </c>
     </row>
@@ -25412,7 +25412,7 @@
         </is>
       </c>
       <c r="C5" s="41" t="n">
-        <v>24603</v>
+        <v>24899</v>
       </c>
       <c r="D5" s="28" t="n">
         <v>131</v>
@@ -25424,10 +25424,10 @@
         <v>131</v>
       </c>
       <c r="G5" s="28" t="n">
-        <v>24130</v>
+        <v>24426</v>
       </c>
       <c r="H5" s="42" t="n">
-        <v>1.922529772791936</v>
+        <v>1.899674685730351</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">

</xml_diff>

<commit_message>
Regenerate all 8 workbooks on 42.6k universe + fix NaN int cast
- Re-ran enrich chain on the widened 42,600-name master (fill_gaps +
  derive + enrich + archetype_tags), multi-archetype names 7,188.
- Regenerated all 8 workbooks; verified 0 nan/inf cells.
- Fixed top_n_by_country NaN->int crash: 'int(x or 0)' returns nan when
  x is NaN (nan is truthy), now guarded with pd.notna. Surfaced once the
  unenriched FDB-expansion names entered the top-30 country slices.
</commit_message>
<xml_diff>
--- a/asymmetry_harvard_workbook.xlsx
+++ b/asymmetry_harvard_workbook.xlsx
@@ -1,67 +1,67 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Index" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_088910_KQ" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_AWC_SI" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_2230_HK" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_0057_HK" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_003650_KS" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_ZENIFIB_BO" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_ALGEV_PA" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_0882_HK" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_TPP_BK" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_SHRIDINE_BO" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_6155_T" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_0100_KL" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_IRC_BK" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_LSIP_JK" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_JAMESWARREN_BO" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_2348_HK" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_4301_T" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_S23_SI" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19_4629_T" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20_1798_T" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21_6907_T" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22_FPIP_ST" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="23_014570_KQ" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="24_TCID_JK" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25_NPK_BK" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26_052330_KQ" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="27_HTMEDIA_BO" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="28_120240_KQ" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="29_6986_T" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="30_035610_KQ" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="31_0114_HK" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="32_7722_T" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="33_BENGALT_BO" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="34_SIAM_BK" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="35_036190_KQ" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="36_PRIMEPRO_BO" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="37_IGAR_JK" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="38_METCO_BK" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="39_0420_HK" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="40_2033_HK" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="41_031510_KQ" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="42_0538_HK" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="43_0212_HK" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="44_1795_T" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="45_047820_KQ" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="46_PBMPOLY_BO" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="47_054800_KQ" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="48_0887_HK" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="49_015230_KS" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50_7219_T" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Methodology" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Index" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="01_088910_KQ" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="02_AWC_SI" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="03_2230_HK" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="04_0057_HK" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="05_003650_KS" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="06_ZENIFIB_BO" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="07_ALGEV_PA" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="08_0882_HK" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="09_TPP_BK" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="10_SHRIDINE_BO" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="11_6155_T" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="12_0100_KL" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="13_IRC_BK" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="14_LSIP_JK" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="15_JAMESWARREN_BO" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="16_2348_HK" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="17_4301_T" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="18_S23_SI" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="19_4629_T" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="20_1798_T" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="21_6907_T" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="22_FPIP_ST" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="23_014570_KQ" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="24_TCID_JK" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="25_NPK_BK" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="26_052330_KQ" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="27_HTMEDIA_BO" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="28_120240_KQ" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="29_6986_T" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="30_035610_KQ" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="31_0114_HK" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="32_7722_T" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="33_BENGALT_BO" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="34_SIAM_BK" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="35_036190_KQ" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="36_PRIMEPRO_BO" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="37_IGAR_JK" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="38_METCO_BK" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="39_0420_HK" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="40_2033_HK" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="41_031510_KQ" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="42_0538_HK" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="43_0212_HK" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="44_1795_T" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="45_047820_KQ" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="46_PBMPOLY_BO" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="47_054800_KQ" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="48_0887_HK" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="49_015230_KS" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="50_7219_T" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="Coverage" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet name="References" sheetId="55" state="visible" r:id="rId55"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -754,7 +754,7 @@
     <row r="11" ht="24" customHeight="1">
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>24,899</t>
+          <t>26,756</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -764,22 +764,22 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>473</t>
+          <t>480</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>133</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>214</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>24,426</t>
+          <t>26,276</t>
         </is>
       </c>
     </row>
@@ -796,7 +796,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>1.9% of universe</t>
+          <t>1.8% of universe</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -833,7 +833,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>This workbook documents the top 50 names from a global universe of 24,899 equities ranked by an entry-today asymmetry score. The upside leg weights factors Anna Yartseva (CAFE WP 33, 2025) finds predictive of 10-bagger outcomes — FCF yield, book-to-market, small size, profitability level, asset-growth gate, contra-momentum. The downside floor leg combines Graham net-net, cash &gt; EV, sub-book and negative-EV signals. Each candidate has been qualitatively reviewed and assigned a verdict of GREEN (high-conviction), YELLOW (risk-flagged), RED (avoid) or UNRESEARCHED. Sheets sequence as Cover, Methodology, Index, per-name pages, Coverage, References.</t>
+          <t>This workbook documents the top 50 names from a global universe of 26,756 equities ranked by an entry-today asymmetry score. The upside leg weights factors Anna Yartseva (CAFE WP 33, 2025) finds predictive of 10-bagger outcomes — FCF yield, book-to-market, small size, profitability level, asset-growth gate, contra-momentum. The downside floor leg combines Graham net-net, cash &gt; EV, sub-book and negative-EV signals. Each candidate has been qualitatively reviewed and assigned a verdict of GREEN (high-conviction), YELLOW (risk-flagged), RED (avoid) or UNRESEARCHED. Sheets sequence as Cover, Methodology, Index, per-name pages, Coverage, References.</t>
         </is>
       </c>
     </row>
@@ -25412,22 +25412,22 @@
         </is>
       </c>
       <c r="C5" s="41" t="n">
-        <v>24899</v>
+        <v>26756</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="F5" s="28" t="n">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="G5" s="28" t="n">
-        <v>24426</v>
+        <v>26276</v>
       </c>
       <c r="H5" s="42" t="n">
-        <v>1.899674685730351</v>
+        <v>1.793990133054268</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">

</xml_diff>

<commit_message>
Deep enrichment complete: merge + regenerate all workbooks
</commit_message>
<xml_diff>
--- a/asymmetry_harvard_workbook.xlsx
+++ b/asymmetry_harvard_workbook.xlsx
@@ -754,7 +754,7 @@
     <row r="11" ht="24" customHeight="1">
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>26,756</t>
+          <t>30,308</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>26,276</t>
+          <t>29,828</t>
         </is>
       </c>
     </row>
@@ -796,7 +796,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>1.8% of universe</t>
+          <t>1.6% of universe</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -833,7 +833,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>This workbook documents the top 50 names from a global universe of 26,756 equities ranked by an entry-today asymmetry score. The upside leg weights factors Anna Yartseva (CAFE WP 33, 2025) finds predictive of 10-bagger outcomes — FCF yield, book-to-market, small size, profitability level, asset-growth gate, contra-momentum. The downside floor leg combines Graham net-net, cash &gt; EV, sub-book and negative-EV signals. Each candidate has been qualitatively reviewed and assigned a verdict of GREEN (high-conviction), YELLOW (risk-flagged), RED (avoid) or UNRESEARCHED. Sheets sequence as Cover, Methodology, Index, per-name pages, Coverage, References.</t>
+          <t>This workbook documents the top 50 names from a global universe of 30,308 equities ranked by an entry-today asymmetry score. The upside leg weights factors Anna Yartseva (CAFE WP 33, 2025) finds predictive of 10-bagger outcomes — FCF yield, book-to-market, small size, profitability level, asset-growth gate, contra-momentum. The downside floor leg combines Graham net-net, cash &gt; EV, sub-book and negative-EV signals. Each candidate has been qualitatively reviewed and assigned a verdict of GREEN (high-conviction), YELLOW (risk-flagged), RED (avoid) or UNRESEARCHED. Sheets sequence as Cover, Methodology, Index, per-name pages, Coverage, References.</t>
         </is>
       </c>
     </row>
@@ -12884,8 +12884,10 @@
           <t>P/E</t>
         </is>
       </c>
-      <c r="C31" s="21" t="n">
-        <v>2215</v>
+      <c r="C31" s="34" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="D31" s="30" t="inlineStr">
         <is>
@@ -25412,7 +25414,7 @@
         </is>
       </c>
       <c r="C5" s="41" t="n">
-        <v>26756</v>
+        <v>30308</v>
       </c>
       <c r="D5" s="28" t="n">
         <v>133</v>
@@ -25424,10 +25426,10 @@
         <v>133</v>
       </c>
       <c r="G5" s="28" t="n">
-        <v>26276</v>
+        <v>29828</v>
       </c>
       <c r="H5" s="42" t="n">
-        <v>1.793990133054268</v>
+        <v>1.583740266596278</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">

</xml_diff>

<commit_message>
Full render: div yield, display dedup, repaired currencies + lynch data
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/asymmetry_harvard_workbook.xlsx
+++ b/asymmetry_harvard_workbook.xlsx
@@ -756,7 +756,7 @@
     <row r="11" ht="24" customHeight="1">
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>25,466</t>
+          <t>25,849</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -766,22 +766,22 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>382</t>
+          <t>394</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>118</t>
+          <t>121</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>169</t>
+          <t>177</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>25,084</t>
+          <t>25,455</t>
         </is>
       </c>
     </row>
@@ -835,7 +835,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>This workbook documents the top 50 names from a global universe of 25,466 equities ranked by an entry-today asymmetry score. The upside leg weights factors Anna Yartseva (CAFE WP 33, 2025) finds predictive of 10-bagger outcomes — FCF yield, book-to-market, small size, profitability level, asset-growth gate, contra-momentum. The downside floor leg combines Graham net-net, cash &gt; EV, sub-book and negative-EV signals. Each candidate has been qualitatively reviewed and assigned a verdict of GREEN (high-conviction), YELLOW (risk-flagged), RED (avoid) or UNRESEARCHED. Sheets sequence as Cover, Methodology, Index, per-name pages, Coverage, References.</t>
+          <t>This workbook documents the top 50 names from a global universe of 25,849 equities ranked by an entry-today asymmetry score. The upside leg weights factors Anna Yartseva (CAFE WP 33, 2025) finds predictive of 10-bagger outcomes — FCF yield, book-to-market, small size, profitability level, asset-growth gate, contra-momentum. The downside floor leg combines Graham net-net, cash &gt; EV, sub-book and negative-EV signals. Each candidate has been qualitatively reviewed and assigned a verdict of GREEN (high-conviction), YELLOW (risk-flagged), RED (avoid) or UNRESEARCHED. Sheets sequence as Cover, Methodology, Index, per-name pages, Coverage, References.</t>
         </is>
       </c>
     </row>
@@ -26053,22 +26053,22 @@
         </is>
       </c>
       <c r="C5" s="41" t="n">
-        <v>25466</v>
+        <v>25849</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E5" s="31" t="n">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="F5" s="31" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G5" s="31" t="n">
-        <v>25084</v>
+        <v>25455</v>
       </c>
       <c r="H5" s="42" t="n">
-        <v>1.500039268043666</v>
+        <v>1.524236914387404</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">

</xml_diff>

<commit_message>
Full render on demand: all 16 books, Lynch coverage 25962 names
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/asymmetry_harvard_workbook.xlsx
+++ b/asymmetry_harvard_workbook.xlsx
@@ -756,7 +756,7 @@
     <row r="11" ht="24" customHeight="1">
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>25,862</t>
+          <t>25,849</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -766,12 +766,12 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>395</t>
+          <t>394</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>122</t>
+          <t>121</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>25,467</t>
+          <t>25,455</t>
         </is>
       </c>
     </row>
@@ -835,7 +835,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>This workbook documents the top 50 names from a global universe of 25,862 equities ranked by an entry-today asymmetry score. The upside leg weights factors Anna Yartseva (CAFE WP 33, 2025) finds predictive of 10-bagger outcomes — FCF yield, book-to-market, small size, profitability level, asset-growth gate, contra-momentum. The downside floor leg combines Graham net-net, cash &gt; EV, sub-book and negative-EV signals. Each candidate has been qualitatively reviewed and assigned a verdict of GREEN (high-conviction), YELLOW (risk-flagged), RED (avoid) or UNRESEARCHED. Sheets sequence as Cover, Methodology, Index, per-name pages, Coverage, References.</t>
+          <t>This workbook documents the top 50 names from a global universe of 25,849 equities ranked by an entry-today asymmetry score. The upside leg weights factors Anna Yartseva (CAFE WP 33, 2025) finds predictive of 10-bagger outcomes — FCF yield, book-to-market, small size, profitability level, asset-growth gate, contra-momentum. The downside floor leg combines Graham net-net, cash &gt; EV, sub-book and negative-EV signals. Each candidate has been qualitatively reviewed and assigned a verdict of GREEN (high-conviction), YELLOW (risk-flagged), RED (avoid) or UNRESEARCHED. Sheets sequence as Cover, Methodology, Index, per-name pages, Coverage, References.</t>
         </is>
       </c>
     </row>
@@ -26055,10 +26055,10 @@
         </is>
       </c>
       <c r="C5" s="41" t="n">
-        <v>25862</v>
+        <v>25849</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E5" s="31" t="n">
         <v>177</v>
@@ -26067,10 +26067,10 @@
         <v>96</v>
       </c>
       <c r="G5" s="31" t="n">
-        <v>25467</v>
+        <v>25455</v>
       </c>
       <c r="H5" s="42" t="n">
-        <v>1.527337406233083</v>
+        <v>1.524236914387404</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">

</xml_diff>

<commit_message>
OTC deep enrichment complete: merge + regenerate all books
</commit_message>
<xml_diff>
--- a/asymmetry_harvard_workbook.xlsx
+++ b/asymmetry_harvard_workbook.xlsx
@@ -756,7 +756,7 @@
     <row r="11" ht="24" customHeight="1">
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>25,849</t>
+          <t>25,862</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -766,12 +766,12 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>394</t>
+          <t>395</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>121</t>
+          <t>122</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>25,455</t>
+          <t>25,467</t>
         </is>
       </c>
     </row>
@@ -835,7 +835,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>This workbook documents the top 50 names from a global universe of 25,849 equities ranked by an entry-today asymmetry score. The upside leg weights factors Anna Yartseva (CAFE WP 33, 2025) finds predictive of 10-bagger outcomes — FCF yield, book-to-market, small size, profitability level, asset-growth gate, contra-momentum. The downside floor leg combines Graham net-net, cash &gt; EV, sub-book and negative-EV signals. Each candidate has been qualitatively reviewed and assigned a verdict of GREEN (high-conviction), YELLOW (risk-flagged), RED (avoid) or UNRESEARCHED. Sheets sequence as Cover, Methodology, Index, per-name pages, Coverage, References.</t>
+          <t>This workbook documents the top 50 names from a global universe of 25,862 equities ranked by an entry-today asymmetry score. The upside leg weights factors Anna Yartseva (CAFE WP 33, 2025) finds predictive of 10-bagger outcomes — FCF yield, book-to-market, small size, profitability level, asset-growth gate, contra-momentum. The downside floor leg combines Graham net-net, cash &gt; EV, sub-book and negative-EV signals. Each candidate has been qualitatively reviewed and assigned a verdict of GREEN (high-conviction), YELLOW (risk-flagged), RED (avoid) or UNRESEARCHED. Sheets sequence as Cover, Methodology, Index, per-name pages, Coverage, References.</t>
         </is>
       </c>
     </row>
@@ -26055,10 +26055,10 @@
         </is>
       </c>
       <c r="C5" s="41" t="n">
-        <v>25849</v>
+        <v>25862</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E5" s="31" t="n">
         <v>177</v>
@@ -26067,10 +26067,10 @@
         <v>96</v>
       </c>
       <c r="G5" s="31" t="n">
-        <v>25455</v>
+        <v>25467</v>
       </c>
       <c r="H5" s="42" t="n">
-        <v>1.524236914387404</v>
+        <v>1.527337406233083</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">

</xml_diff>

<commit_message>
Full render: all books on 80 archetypes incl. Biotech Deep Value
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/asymmetry_harvard_workbook.xlsx
+++ b/asymmetry_harvard_workbook.xlsx
@@ -24,14 +24,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_TPP_BK" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_LSIP_JK" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_120240_KQ" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_035610_KQ" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_3798_HK" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_3798_HK" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_035610_KQ" sheetId="19" state="visible" r:id="rId19"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_031510_KQ" sheetId="20" state="visible" r:id="rId20"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_052330_KQ" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19_KROS" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20_348350_KQ" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21_2348_HK" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22_METCO_BK" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19_348350_KQ" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20_2348_HK" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21_METCO_BK" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22_KROS" sheetId="25" state="visible" r:id="rId25"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="23_S23_SI" sheetId="26" state="visible" r:id="rId26"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="24_095660_KQ" sheetId="27" state="visible" r:id="rId27"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25_051160_KQ" sheetId="28" state="visible" r:id="rId28"/>
@@ -4815,6 +4815,488 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>#15    3798.HK    Homeland Interactive Technology Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="4" customHeight="1">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="B3" s="26" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="C3" s="37" t="inlineStr">
+        <is>
+          <t>UNRESEARCHED</t>
+        </is>
+      </c>
+      <c r="D3" s="26" t="inlineStr">
+        <is>
+          <t>Entry-today score</t>
+        </is>
+      </c>
+      <c r="E3" s="28" t="n">
+        <v>1.146428117925815</v>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SNAPSHOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="B6" s="30" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t>Interactive Media &amp; Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>Bucket</t>
+        </is>
+      </c>
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t>Small Cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t>Market cap (USD)</t>
+        </is>
+      </c>
+      <c r="B10" s="31" t="n">
+        <v>193180522.7553062</v>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>Revenue TTM (USD)</t>
+        </is>
+      </c>
+      <c r="B11" s="31" t="n">
+        <v>172106635.0032687</v>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
+          <t>As-of</t>
+        </is>
+      </c>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>INVESTMENT THESIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="B15" s="32" t="inlineStr">
+        <is>
+          <t>Unresearched. No qualitative thesis on file; ranking driven entirely by quantitative signals (see Score decomposition below).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1"/>
+    <row r="17" ht="22" customHeight="1"/>
+    <row r="18" ht="22" customHeight="1"/>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>SCORE DECOMPOSITION</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="B21" s="33" t="inlineStr">
+        <is>
+          <t>Asymmetry (raw)</t>
+        </is>
+      </c>
+      <c r="C21" s="22" t="n">
+        <v>0.6573455939461111</v>
+      </c>
+      <c r="D21" s="33" t="inlineStr">
+        <is>
+          <t>Intrinsic discount</t>
+        </is>
+      </c>
+      <c r="E21" s="22" t="n">
+        <v>0.5915588255881016</v>
+      </c>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="B22" s="33" t="inlineStr">
+        <is>
+          <t>Upside leg</t>
+        </is>
+      </c>
+      <c r="C22" s="22" t="n">
+        <v>0.5617341988444753</v>
+      </c>
+      <c r="D22" s="33" t="inlineStr">
+        <is>
+          <t>Qual multiplier (x)</t>
+        </is>
+      </c>
+      <c r="E22" s="22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="B23" s="33" t="inlineStr">
+        <is>
+          <t>Downside floor</t>
+        </is>
+      </c>
+      <c r="C23" s="22" t="n">
+        <v>0.7692307692307692</v>
+      </c>
+      <c r="D23" s="33" t="inlineStr">
+        <is>
+          <t>Post-rally factor (x)</t>
+        </is>
+      </c>
+      <c r="E23" s="22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="B24" s="33" t="inlineStr">
+        <is>
+          <t>Yartseva composite</t>
+        </is>
+      </c>
+      <c r="C24" s="22" t="n">
+        <v>0.8495485218474618</v>
+      </c>
+      <c r="D24" s="33" t="inlineStr">
+        <is>
+          <t>Confirmation (x)</t>
+        </is>
+      </c>
+      <c r="E24" s="22" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="B25" s="33" t="inlineStr">
+        <is>
+          <t>Berezin growth</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="n">
+        <v>0.4128425191777984</v>
+      </c>
+      <c r="D25" s="33" t="inlineStr">
+        <is>
+          <t>Cluster signals (of 7)</t>
+        </is>
+      </c>
+      <c r="E25" s="34" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>VALUATION &amp; BALANCE SHEET</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>P/B</t>
+        </is>
+      </c>
+      <c r="C28" s="22" t="n">
+        <v>0.63482887</v>
+      </c>
+      <c r="D28" s="33" t="inlineStr">
+        <is>
+          <t>NCAV / mcap (%)</t>
+        </is>
+      </c>
+      <c r="E28" s="25" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="16" customHeight="1">
+      <c r="B29" s="33" t="inlineStr">
+        <is>
+          <t>EV / EBITDA</t>
+        </is>
+      </c>
+      <c r="C29" s="22" t="n">
+        <v>1.119</v>
+      </c>
+      <c r="D29" s="33" t="inlineStr">
+        <is>
+          <t>Net debt / EBITDA (x)</t>
+        </is>
+      </c>
+      <c r="E29" s="22" t="n">
+        <v>-7.225898256848096</v>
+      </c>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="B30" s="33" t="inlineStr">
+        <is>
+          <t>EV / EBIT</t>
+        </is>
+      </c>
+      <c r="C30" s="22" t="n">
+        <v>2.041767239331802</v>
+      </c>
+      <c r="D30" s="33" t="inlineStr">
+        <is>
+          <t>ROCE (%)</t>
+        </is>
+      </c>
+      <c r="E30" s="23" t="n">
+        <v>33.75755216989689</v>
+      </c>
+    </row>
+    <row r="31" ht="16" customHeight="1">
+      <c r="B31" s="33" t="inlineStr">
+        <is>
+          <t>P/E</t>
+        </is>
+      </c>
+      <c r="C31" s="22" t="n">
+        <v>20.000002</v>
+      </c>
+      <c r="D31" s="33" t="inlineStr">
+        <is>
+          <t>EBITDA margin (%)</t>
+        </is>
+      </c>
+      <c r="E31" s="23" t="n">
+        <v>13.1301770234321</v>
+      </c>
+    </row>
+    <row r="32" ht="16" customHeight="1">
+      <c r="B32" s="33" t="inlineStr">
+        <is>
+          <t>P/S</t>
+        </is>
+      </c>
+      <c r="C32" s="22" t="n">
+        <v>1.2164296</v>
+      </c>
+      <c r="D32" s="33" t="inlineStr">
+        <is>
+          <t>Insider ownership (%)</t>
+        </is>
+      </c>
+      <c r="E32" s="23" t="n">
+        <v>74.694</v>
+      </c>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="B33" s="33" t="inlineStr">
+        <is>
+          <t>FCF yield (%)</t>
+        </is>
+      </c>
+      <c r="C33" s="23" t="n">
+        <v>11.29592044426044</v>
+      </c>
+      <c r="D33" s="33" t="inlineStr">
+        <is>
+          <t>Rev 3y CAGR (%)</t>
+        </is>
+      </c>
+      <c r="E33" s="25" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="16" customHeight="1">
+      <c r="B34" s="33" t="inlineStr">
+        <is>
+          <t>Net cash / mcap (%)</t>
+        </is>
+      </c>
+      <c r="C34" s="23" t="n">
+        <v>72.84153319603385</v>
+      </c>
+      <c r="D34" s="33" t="inlineStr">
+        <is>
+          <t>Rev YoY (TTM, %)</t>
+        </is>
+      </c>
+      <c r="E34" s="23" t="n">
+        <v>-2.6933510331294</v>
+      </c>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="B35" s="33" t="inlineStr">
+        <is>
+          <t>Cash / EV (x)</t>
+        </is>
+      </c>
+      <c r="C35" s="22" t="n">
+        <v>3.142024571801568</v>
+      </c>
+      <c r="D35" s="33" t="inlineStr">
+        <is>
+          <t>12m price momentum (%)</t>
+        </is>
+      </c>
+      <c r="E35" s="23" t="n">
+        <v>-18.09</v>
+      </c>
+    </row>
+    <row r="37" ht="16" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>SIGNALS FIRING</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="16" customHeight="1">
+      <c r="B38" s="35" t="inlineStr">
+        <is>
+          <t>·  Cash &gt; EV  (downside floor in place)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="16" customHeight="1">
+      <c r="B39" s="35" t="inlineStr">
+        <is>
+          <t>·  Sub-book  (P/B 0.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="16" customHeight="1">
+      <c r="B40" s="35" t="inlineStr">
+        <is>
+          <t>·  Insider-aligned  (75% insider)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="16" customHeight="1">
+      <c r="B41" s="35" t="inlineStr">
+        <is>
+          <t>·  Cluster stack  (6 of 7 inflection signals)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="36" t="n"/>
+      <c r="B43" s="36" t="n"/>
+      <c r="C43" s="36" t="n"/>
+      <c r="D43" s="36" t="n"/>
+      <c r="E43" s="36" t="n"/>
+      <c r="F43" s="36" t="n"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="26" t="inlineStr">
+        <is>
+          <t>Asymmetry Workbook  ·  Sheet 15 of 50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="B15:E18"/>
+    <mergeCell ref="A27:E27"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00707070"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4829,7 +5311,7 @@
     <row r="1" ht="20" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>#15    035610.KQ    Solborn, Inc.</t>
+          <t>#16    035610.KQ    Solborn, Inc.</t>
         </is>
       </c>
     </row>
@@ -4858,7 +5340,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.146648181877715</v>
+        <v>1.137221610175333</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -5039,7 +5521,7 @@
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>1.2164</v>
+        <v>1.2064</v>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
@@ -5119,8 +5601,10 @@
           <t>ROCE (%)</t>
         </is>
       </c>
-      <c r="E30" s="23" t="n">
-        <v>197.6613890777809</v>
+      <c r="E30" s="25" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
@@ -5279,7 +5763,7 @@
     <row r="50">
       <c r="B50" s="26" t="inlineStr">
         <is>
-          <t>Asymmetry Workbook  ·  Sheet 15 of 50</t>
+          <t>Asymmetry Workbook  ·  Sheet 16 of 50</t>
         </is>
       </c>
     </row>
@@ -5300,488 +5784,6 @@
     <mergeCell ref="A37:E37"/>
     <mergeCell ref="B39:E39"/>
     <mergeCell ref="B44:E46"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="B15:E18"/>
-    <mergeCell ref="A27:E27"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00707070"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F44"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="4" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>#16    3798.HK    Homeland Interactive Technology Ltd.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="4" customHeight="1">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="B3" s="26" t="inlineStr">
-        <is>
-          <t>Verdict</t>
-        </is>
-      </c>
-      <c r="C3" s="37" t="inlineStr">
-        <is>
-          <t>UNRESEARCHED</t>
-        </is>
-      </c>
-      <c r="D3" s="26" t="inlineStr">
-        <is>
-          <t>Entry-today score</t>
-        </is>
-      </c>
-      <c r="E3" s="28" t="n">
-        <v>1.146428117925815</v>
-      </c>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>SNAPSHOT</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="29" t="inlineStr">
-        <is>
-          <t>Country</t>
-        </is>
-      </c>
-      <c r="B6" s="30" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="29" t="inlineStr">
-        <is>
-          <t>Sector</t>
-        </is>
-      </c>
-      <c r="B7" s="30" t="inlineStr">
-        <is>
-          <t>Communication Services</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="29" t="inlineStr">
-        <is>
-          <t>Industry</t>
-        </is>
-      </c>
-      <c r="B8" s="30" t="inlineStr">
-        <is>
-          <t>Interactive Media &amp; Services</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="29" t="inlineStr">
-        <is>
-          <t>Bucket</t>
-        </is>
-      </c>
-      <c r="B9" s="30" t="inlineStr">
-        <is>
-          <t>Small Cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="29" t="inlineStr">
-        <is>
-          <t>Market cap (USD)</t>
-        </is>
-      </c>
-      <c r="B10" s="31" t="n">
-        <v>193180522.7553062</v>
-      </c>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="29" t="inlineStr">
-        <is>
-          <t>Revenue TTM (USD)</t>
-        </is>
-      </c>
-      <c r="B11" s="31" t="n">
-        <v>172106635.0032687</v>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="29" t="inlineStr">
-        <is>
-          <t>As-of</t>
-        </is>
-      </c>
-      <c r="B12" s="30" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>INVESTMENT THESIS</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="32" t="inlineStr">
-        <is>
-          <t>Unresearched. No qualitative thesis on file; ranking driven entirely by quantitative signals (see Score decomposition below).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1"/>
-    <row r="17" ht="22" customHeight="1"/>
-    <row r="18" ht="22" customHeight="1"/>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>SCORE DECOMPOSITION</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="B21" s="33" t="inlineStr">
-        <is>
-          <t>Asymmetry (raw)</t>
-        </is>
-      </c>
-      <c r="C21" s="22" t="n">
-        <v>0.6573455939461111</v>
-      </c>
-      <c r="D21" s="33" t="inlineStr">
-        <is>
-          <t>Intrinsic discount</t>
-        </is>
-      </c>
-      <c r="E21" s="22" t="n">
-        <v>0.5915588255881016</v>
-      </c>
-    </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="B22" s="33" t="inlineStr">
-        <is>
-          <t>Upside leg</t>
-        </is>
-      </c>
-      <c r="C22" s="22" t="n">
-        <v>0.5617341988444753</v>
-      </c>
-      <c r="D22" s="33" t="inlineStr">
-        <is>
-          <t>Qual multiplier (x)</t>
-        </is>
-      </c>
-      <c r="E22" s="22" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="B23" s="33" t="inlineStr">
-        <is>
-          <t>Downside floor</t>
-        </is>
-      </c>
-      <c r="C23" s="22" t="n">
-        <v>0.7692307692307692</v>
-      </c>
-      <c r="D23" s="33" t="inlineStr">
-        <is>
-          <t>Post-rally factor (x)</t>
-        </is>
-      </c>
-      <c r="E23" s="22" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="B24" s="33" t="inlineStr">
-        <is>
-          <t>Yartseva composite</t>
-        </is>
-      </c>
-      <c r="C24" s="22" t="n">
-        <v>0.8495485218474618</v>
-      </c>
-      <c r="D24" s="33" t="inlineStr">
-        <is>
-          <t>Confirmation (x)</t>
-        </is>
-      </c>
-      <c r="E24" s="22" t="n">
-        <v>1.3</v>
-      </c>
-    </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="B25" s="33" t="inlineStr">
-        <is>
-          <t>Berezin growth</t>
-        </is>
-      </c>
-      <c r="C25" s="22" t="n">
-        <v>0.4128425191777984</v>
-      </c>
-      <c r="D25" s="33" t="inlineStr">
-        <is>
-          <t>Cluster signals (of 7)</t>
-        </is>
-      </c>
-      <c r="E25" s="34" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>VALUATION &amp; BALANCE SHEET</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="16" customHeight="1">
-      <c r="B28" s="33" t="inlineStr">
-        <is>
-          <t>P/B</t>
-        </is>
-      </c>
-      <c r="C28" s="22" t="n">
-        <v>0.63482887</v>
-      </c>
-      <c r="D28" s="33" t="inlineStr">
-        <is>
-          <t>NCAV / mcap (%)</t>
-        </is>
-      </c>
-      <c r="E28" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="16" customHeight="1">
-      <c r="B29" s="33" t="inlineStr">
-        <is>
-          <t>EV / EBITDA</t>
-        </is>
-      </c>
-      <c r="C29" s="22" t="n">
-        <v>1.119</v>
-      </c>
-      <c r="D29" s="33" t="inlineStr">
-        <is>
-          <t>Net debt / EBITDA (x)</t>
-        </is>
-      </c>
-      <c r="E29" s="22" t="n">
-        <v>-7.225898256848096</v>
-      </c>
-    </row>
-    <row r="30" ht="16" customHeight="1">
-      <c r="B30" s="33" t="inlineStr">
-        <is>
-          <t>EV / EBIT</t>
-        </is>
-      </c>
-      <c r="C30" s="22" t="n">
-        <v>2.041767239331802</v>
-      </c>
-      <c r="D30" s="33" t="inlineStr">
-        <is>
-          <t>ROCE (%)</t>
-        </is>
-      </c>
-      <c r="E30" s="23" t="n">
-        <v>33.75755216989689</v>
-      </c>
-    </row>
-    <row r="31" ht="16" customHeight="1">
-      <c r="B31" s="33" t="inlineStr">
-        <is>
-          <t>P/E</t>
-        </is>
-      </c>
-      <c r="C31" s="22" t="n">
-        <v>20.000002</v>
-      </c>
-      <c r="D31" s="33" t="inlineStr">
-        <is>
-          <t>EBITDA margin (%)</t>
-        </is>
-      </c>
-      <c r="E31" s="23" t="n">
-        <v>13.1301770234321</v>
-      </c>
-    </row>
-    <row r="32" ht="16" customHeight="1">
-      <c r="B32" s="33" t="inlineStr">
-        <is>
-          <t>P/S</t>
-        </is>
-      </c>
-      <c r="C32" s="22" t="n">
-        <v>1.2164296</v>
-      </c>
-      <c r="D32" s="33" t="inlineStr">
-        <is>
-          <t>Insider ownership (%)</t>
-        </is>
-      </c>
-      <c r="E32" s="23" t="n">
-        <v>74.694</v>
-      </c>
-    </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="B33" s="33" t="inlineStr">
-        <is>
-          <t>FCF yield (%)</t>
-        </is>
-      </c>
-      <c r="C33" s="23" t="n">
-        <v>11.29592044426044</v>
-      </c>
-      <c r="D33" s="33" t="inlineStr">
-        <is>
-          <t>Rev 3y CAGR (%)</t>
-        </is>
-      </c>
-      <c r="E33" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="B34" s="33" t="inlineStr">
-        <is>
-          <t>Net cash / mcap (%)</t>
-        </is>
-      </c>
-      <c r="C34" s="23" t="n">
-        <v>72.84153319603385</v>
-      </c>
-      <c r="D34" s="33" t="inlineStr">
-        <is>
-          <t>Rev YoY (TTM, %)</t>
-        </is>
-      </c>
-      <c r="E34" s="23" t="n">
-        <v>-2.6933510331294</v>
-      </c>
-    </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="B35" s="33" t="inlineStr">
-        <is>
-          <t>Cash / EV (x)</t>
-        </is>
-      </c>
-      <c r="C35" s="22" t="n">
-        <v>3.142024571801568</v>
-      </c>
-      <c r="D35" s="33" t="inlineStr">
-        <is>
-          <t>12m price momentum (%)</t>
-        </is>
-      </c>
-      <c r="E35" s="23" t="n">
-        <v>-18.09</v>
-      </c>
-    </row>
-    <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>SIGNALS FIRING</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="16" customHeight="1">
-      <c r="B38" s="35" t="inlineStr">
-        <is>
-          <t>·  Cash &gt; EV  (downside floor in place)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="16" customHeight="1">
-      <c r="B39" s="35" t="inlineStr">
-        <is>
-          <t>·  Sub-book  (P/B 0.63)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="16" customHeight="1">
-      <c r="B40" s="35" t="inlineStr">
-        <is>
-          <t>·  Insider-aligned  (75% insider)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="16" customHeight="1">
-      <c r="B41" s="35" t="inlineStr">
-        <is>
-          <t>·  Cluster stack  (6 of 7 inflection signals)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="36" t="n"/>
-      <c r="B43" s="36" t="n"/>
-      <c r="C43" s="36" t="n"/>
-      <c r="D43" s="36" t="n"/>
-      <c r="E43" s="36" t="n"/>
-      <c r="F43" s="36" t="n"/>
-    </row>
-    <row r="44">
-      <c r="B44" s="26" t="inlineStr">
-        <is>
-          <t>Asymmetry Workbook  ·  Sheet 16 of 50</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="16">
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="B41:E41"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B38:E38"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A37:E37"/>
-    <mergeCell ref="B39:E39"/>
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="B15:E18"/>
     <mergeCell ref="A27:E27"/>
@@ -6945,7 +6947,7 @@
     <row r="1" ht="20" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>#19    KROS    Keros Therapeutics, Inc.</t>
+          <t>#19    348350.KQ    WITHTECH Co., LTD.</t>
         </is>
       </c>
     </row>
@@ -6974,7 +6976,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.11727586668782</v>
+        <v>1.113650562417347</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -6992,7 +6994,7 @@
       </c>
       <c r="B6" s="30" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KR</t>
         </is>
       </c>
     </row>
@@ -7004,7 +7006,7 @@
       </c>
       <c r="B7" s="30" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
@@ -7014,10 +7016,8 @@
           <t>Industry</t>
         </is>
       </c>
-      <c r="B8" s="30" t="inlineStr">
-        <is>
-          <t>Biotechnology</t>
-        </is>
+      <c r="B8" s="30" t="n">
+        <v/>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
@@ -7028,7 +7028,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Small Cap</t>
+          <t>Large Cap</t>
         </is>
       </c>
     </row>
@@ -7039,7 +7039,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>224443760</v>
+        <v>60858057.77970123</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -7049,7 +7049,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>244061000</v>
+        <v>37014740.95624924</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -7060,7 +7060,7 @@
       </c>
       <c r="B12" s="30" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-03-31</t>
         </is>
       </c>
     </row>
@@ -7095,7 +7095,7 @@
         </is>
       </c>
       <c r="C21" s="22" t="n">
-        <v>0.6305867949791741</v>
+        <v>0.588439175935826</v>
       </c>
       <c r="D21" s="33" t="inlineStr">
         <is>
@@ -7103,7 +7103,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.67887376</v>
+        <v>0.7650282137291016</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -7113,7 +7113,7 @@
         </is>
       </c>
       <c r="C22" s="22" t="n">
-        <v>0.5716070773780287</v>
+        <v>0.5626735786360552</v>
       </c>
       <c r="D22" s="33" t="inlineStr">
         <is>
@@ -7131,7 +7131,7 @@
         </is>
       </c>
       <c r="C23" s="22" t="n">
-        <v>0.6956521739130435</v>
+        <v>0.6153846153846153</v>
       </c>
       <c r="D23" s="33" t="inlineStr">
         <is>
@@ -7149,7 +7149,7 @@
         </is>
       </c>
       <c r="C24" s="22" t="n">
-        <v>0.837901</v>
+        <v>0.694261</v>
       </c>
       <c r="D24" s="33" t="inlineStr">
         <is>
@@ -7157,7 +7157,7 @@
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>1.24</v>
+        <v>1.2617</v>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
@@ -7167,7 +7167,7 @@
         </is>
       </c>
       <c r="C25" s="22" t="n">
-        <v>0.4395225067843441</v>
+        <v>0.467269358229353</v>
       </c>
       <c r="D25" s="33" t="inlineStr">
         <is>
@@ -7175,7 +7175,7 @@
         </is>
       </c>
       <c r="E25" s="34" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
@@ -7192,7 +7192,7 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.8556312</v>
+        <v>0.7937623623751395</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
@@ -7200,7 +7200,7 @@
         </is>
       </c>
       <c r="E28" s="23" t="n">
-        <v>127.0432475398032</v>
+        <v>75.63918384940335</v>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
@@ -7210,7 +7210,7 @@
         </is>
       </c>
       <c r="C29" s="22" t="n">
-        <v>0.18</v>
+        <v>1.723</v>
       </c>
       <c r="D29" s="33" t="inlineStr">
         <is>
@@ -7218,7 +7218,7 @@
         </is>
       </c>
       <c r="E29" s="22" t="n">
-        <v>-3.916326471524943</v>
+        <v>-4.466251897016345</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
@@ -7227,10 +7227,8 @@
           <t>EV / EBIT</t>
         </is>
       </c>
-      <c r="C30" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="C30" s="22" t="n">
+        <v>2.795730826372435</v>
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
@@ -7238,7 +7236,7 @@
         </is>
       </c>
       <c r="E30" s="23" t="n">
-        <v>207.2668711656441</v>
+        <v>6.48271546413415</v>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
@@ -7258,7 +7256,7 @@
         </is>
       </c>
       <c r="E31" s="23" t="n">
-        <v>28.30357984274423</v>
+        <v>24.38145444513379</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
@@ -7268,7 +7266,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>14.948965</v>
+        <v>1.4497193</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -7276,7 +7274,7 @@
         </is>
       </c>
       <c r="E32" s="23" t="n">
-        <v>3.641</v>
+        <v>57.577</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
@@ -7286,7 +7284,7 @@
         </is>
       </c>
       <c r="C33" s="23" t="n">
-        <v>36.66783771232035</v>
+        <v>9.770428543556529</v>
       </c>
       <c r="D33" s="33" t="inlineStr">
         <is>
@@ -7306,7 +7304,7 @@
         </is>
       </c>
       <c r="C34" s="23" t="n">
-        <v>135.4560479850007</v>
+        <v>97.41201443595627</v>
       </c>
       <c r="D34" s="33" t="inlineStr">
         <is>
@@ -7314,7 +7312,7 @@
         </is>
       </c>
       <c r="E34" s="23" t="n">
-        <v>6774.957746478873</v>
+        <v>29.74903547376832</v>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
@@ -7323,10 +7321,8 @@
           <t>Cash / EV (x)</t>
         </is>
       </c>
-      <c r="C35" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="C35" s="22" t="n">
+        <v>27.45971875741036</v>
       </c>
       <c r="D35" s="33" t="inlineStr">
         <is>
@@ -7334,7 +7330,7 @@
         </is>
       </c>
       <c r="E35" s="23" t="n">
-        <v>-25.62</v>
+        <v>20.77</v>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1">
@@ -7347,21 +7343,21 @@
     <row r="38" ht="16" customHeight="1">
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>·  Negative enterprise value</t>
+          <t>·  Sub-book  (P/B 0.79)</t>
         </is>
       </c>
     </row>
     <row r="39" ht="16" customHeight="1">
       <c r="B39" s="35" t="inlineStr">
         <is>
-          <t>·  Sub-book  (P/B 0.86)</t>
+          <t>·  Insider-aligned  (58% insider)</t>
         </is>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1">
       <c r="B40" s="35" t="inlineStr">
         <is>
-          <t>·  Cluster stack  (5 of 7 inflection signals)</t>
+          <t>·  Cluster stack  (4 of 7 inflection signals)</t>
         </is>
       </c>
     </row>
@@ -7375,7 +7371,7 @@
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="12" t="inlineStr">
         <is>
-          <t>growth-flip; first-positive: FCF/EBITDA/CFO/NI/ROCE; ROCE improving from &lt;=0; accelerating sales; under-priced vs fundamentals; cash 138% of mcap</t>
+          <t>growth-flip; accelerating sales; under-priced vs fundamentals; cheap+grow (EV/EBIT 2.8x)</t>
         </is>
       </c>
     </row>
@@ -7427,7 +7423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -7441,7 +7437,7 @@
     <row r="1" ht="20" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>#20    348350.KQ    WITHTECH Co., LTD.</t>
+          <t>#20    2348.HK    Dawnrays Pharmaceutical (Holdings) Limited</t>
         </is>
       </c>
     </row>
@@ -7470,7 +7466,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.113650562417347</v>
+        <v>1.09772165902702</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -7488,7 +7484,7 @@
       </c>
       <c r="B6" s="30" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>HK</t>
         </is>
       </c>
     </row>
@@ -7500,7 +7496,7 @@
       </c>
       <c r="B7" s="30" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Health Care</t>
         </is>
       </c>
     </row>
@@ -7510,8 +7506,10 @@
           <t>Industry</t>
         </is>
       </c>
-      <c r="B8" s="30" t="n">
-        <v/>
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t>Pharmaceuticals</t>
+        </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
@@ -7522,7 +7520,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Large Cap</t>
+          <t>Small Cap</t>
         </is>
       </c>
     </row>
@@ -7533,7 +7531,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>60858057.77970123</v>
+        <v>189917124.4803295</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -7543,7 +7541,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>37014740.95624924</v>
+        <v>157064460.8974904</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -7554,7 +7552,7 @@
       </c>
       <c r="B12" s="30" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2025-12-31</t>
         </is>
       </c>
     </row>
@@ -7589,7 +7587,7 @@
         </is>
       </c>
       <c r="C21" s="22" t="n">
-        <v>0.588439175935826</v>
+        <v>0.6098453661261224</v>
       </c>
       <c r="D21" s="33" t="inlineStr">
         <is>
@@ -7597,7 +7595,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.7650282137291016</v>
+        <v>0.9079045322105156</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -7607,7 +7605,7 @@
         </is>
       </c>
       <c r="C22" s="22" t="n">
-        <v>0.5626735786360552</v>
+        <v>0.4834847817611555</v>
       </c>
       <c r="D22" s="33" t="inlineStr">
         <is>
@@ -7625,7 +7623,7 @@
         </is>
       </c>
       <c r="C23" s="22" t="n">
-        <v>0.6153846153846153</v>
+        <v>0.7692307692307692</v>
       </c>
       <c r="D23" s="33" t="inlineStr">
         <is>
@@ -7643,7 +7641,7 @@
         </is>
       </c>
       <c r="C24" s="22" t="n">
-        <v>0.694261</v>
+        <v>0.761567</v>
       </c>
       <c r="D24" s="33" t="inlineStr">
         <is>
@@ -7651,7 +7649,7 @@
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>1.2617</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
@@ -7661,7 +7659,7 @@
         </is>
       </c>
       <c r="C25" s="22" t="n">
-        <v>0.467269358229353</v>
+        <v>0.4269003334734619</v>
       </c>
       <c r="D25" s="33" t="inlineStr">
         <is>
@@ -7686,7 +7684,7 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.7937623623751395</v>
+        <v>0.37188843</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
@@ -7694,7 +7692,7 @@
         </is>
       </c>
       <c r="E28" s="23" t="n">
-        <v>75.63918384940335</v>
+        <v>104.7508519298697</v>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
@@ -7704,7 +7702,7 @@
         </is>
       </c>
       <c r="C29" s="22" t="n">
-        <v>1.723</v>
+        <v>0.2541832540201263</v>
       </c>
       <c r="D29" s="33" t="inlineStr">
         <is>
@@ -7712,7 +7710,7 @@
         </is>
       </c>
       <c r="E29" s="22" t="n">
-        <v>-4.466251897016345</v>
+        <v>-4.049683737461582</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
@@ -7721,8 +7719,10 @@
           <t>EV / EBIT</t>
         </is>
       </c>
-      <c r="C30" s="22" t="n">
-        <v>2.795730826372435</v>
+      <c r="C30" s="25" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
@@ -7730,7 +7730,7 @@
         </is>
       </c>
       <c r="E30" s="23" t="n">
-        <v>6.48271546413415</v>
+        <v>13.2643076741945</v>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
@@ -7739,10 +7739,8 @@
           <t>P/E</t>
         </is>
       </c>
-      <c r="C31" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="C31" s="22" t="n">
+        <v>5.5</v>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
@@ -7750,7 +7748,7 @@
         </is>
       </c>
       <c r="E31" s="23" t="n">
-        <v>24.38145444513379</v>
+        <v>30.0813979089536</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
@@ -7760,7 +7758,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>1.4497193</v>
+        <v>1.2983886</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -7768,7 +7766,7 @@
         </is>
       </c>
       <c r="E32" s="23" t="n">
-        <v>57.577</v>
+        <v>67.661005</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
@@ -7778,7 +7776,7 @@
         </is>
       </c>
       <c r="C33" s="23" t="n">
-        <v>9.770428543556529</v>
+        <v>14.81031382345322</v>
       </c>
       <c r="D33" s="33" t="inlineStr">
         <is>
@@ -7798,7 +7796,7 @@
         </is>
       </c>
       <c r="C34" s="23" t="n">
-        <v>97.41201443595627</v>
+        <v>94.09407273683851</v>
       </c>
       <c r="D34" s="33" t="inlineStr">
         <is>
@@ -7806,7 +7804,7 @@
         </is>
       </c>
       <c r="E34" s="23" t="n">
-        <v>29.74903547376832</v>
+        <v>16.08568822862014</v>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
@@ -7816,7 +7814,7 @@
         </is>
       </c>
       <c r="C35" s="22" t="n">
-        <v>27.45971875741036</v>
+        <v>16.75536368504713</v>
       </c>
       <c r="D35" s="33" t="inlineStr">
         <is>
@@ -7824,7 +7822,7 @@
         </is>
       </c>
       <c r="E35" s="23" t="n">
-        <v>20.77</v>
+        <v>-14.17</v>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1">
@@ -7837,71 +7835,79 @@
     <row r="38" ht="16" customHeight="1">
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>·  Sub-book  (P/B 0.79)</t>
+          <t>·  Cash &gt; EV  (downside floor in place)</t>
         </is>
       </c>
     </row>
     <row r="39" ht="16" customHeight="1">
       <c r="B39" s="35" t="inlineStr">
         <is>
-          <t>·  Insider-aligned  (58% insider)</t>
+          <t>·  Sub-book  (P/B 0.37)</t>
         </is>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1">
       <c r="B40" s="35" t="inlineStr">
         <is>
+          <t>·  Insider-aligned  (68% insider)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="16" customHeight="1">
+      <c r="B41" s="35" t="inlineStr">
+        <is>
           <t>·  Cluster stack  (4 of 7 inflection signals)</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="5" t="inlineStr">
+    <row r="43" ht="16" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>growth-flip; accelerating sales; under-priced vs fundamentals; cheap+grow (EV/EBIT 2.8x)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="18" customHeight="1"/>
+    <row r="44" ht="18" customHeight="1">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>growth-flip; accelerating sales; under-priced vs fundamentals; cheap+grow (EV/EBIT 0.4x); cash 99% of mcap; cash &gt; EV (16.76x, net cash 94% mcap)</t>
+        </is>
+      </c>
+    </row>
     <row r="45" ht="18" customHeight="1"/>
-    <row r="48">
-      <c r="A48" s="36" t="n"/>
-      <c r="B48" s="36" t="n"/>
-      <c r="C48" s="36" t="n"/>
-      <c r="D48" s="36" t="n"/>
-      <c r="E48" s="36" t="n"/>
-      <c r="F48" s="36" t="n"/>
-    </row>
+    <row r="46" ht="18" customHeight="1"/>
     <row r="49">
-      <c r="B49" s="26" t="inlineStr">
+      <c r="A49" s="36" t="n"/>
+      <c r="B49" s="36" t="n"/>
+      <c r="C49" s="36" t="n"/>
+      <c r="D49" s="36" t="n"/>
+      <c r="E49" s="36" t="n"/>
+      <c r="F49" s="36" t="n"/>
+    </row>
+    <row r="50">
+      <c r="B50" s="26" t="inlineStr">
         <is>
           <t>Asymmetry Workbook  ·  Sheet 20 of 50</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="18">
     <mergeCell ref="B40:E40"/>
     <mergeCell ref="B9:E9"/>
+    <mergeCell ref="B41:E41"/>
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A43:E43"/>
     <mergeCell ref="B12:E12"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="B38:E38"/>
-    <mergeCell ref="A42:E42"/>
-    <mergeCell ref="B43:E45"/>
     <mergeCell ref="B7:E7"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A37:E37"/>
     <mergeCell ref="B39:E39"/>
+    <mergeCell ref="B44:E46"/>
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="B15:E18"/>
     <mergeCell ref="A27:E27"/>
@@ -7931,7 +7937,7 @@
     <row r="1" ht="20" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>#21    2348.HK    Dawnrays Pharmaceutical (Holdings) Limited</t>
+          <t>#21    METCO.BK    Muramoto Electron (Thailand) Public Company Limited</t>
         </is>
       </c>
     </row>
@@ -7949,9 +7955,9 @@
           <t>Verdict</t>
         </is>
       </c>
-      <c r="C3" s="37" t="inlineStr">
-        <is>
-          <t>UNRESEARCHED</t>
+      <c r="C3" s="27" t="inlineStr">
+        <is>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="D3" s="26" t="inlineStr">
@@ -7960,7 +7966,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.09772165902702</v>
+        <v>1.095391292032167</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -7978,7 +7984,7 @@
       </c>
       <c r="B6" s="30" t="inlineStr">
         <is>
-          <t>HK</t>
+          <t>TH</t>
         </is>
       </c>
     </row>
@@ -7990,7 +7996,7 @@
       </c>
       <c r="B7" s="30" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Information Technology</t>
         </is>
       </c>
     </row>
@@ -8002,7 +8008,7 @@
       </c>
       <c r="B8" s="30" t="inlineStr">
         <is>
-          <t>Pharmaceuticals</t>
+          <t>Electronic Equipment, Instruments &amp; Components</t>
         </is>
       </c>
     </row>
@@ -8014,7 +8020,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Small Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
     </row>
@@ -8025,7 +8031,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>189917124.4803295</v>
+        <v>189173887.7198486</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -8035,7 +8041,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>157064460.8974904</v>
+        <v>514626167.5263252</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -8046,7 +8052,7 @@
       </c>
       <c r="B12" s="30" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-03-31</t>
         </is>
       </c>
     </row>
@@ -8060,7 +8066,7 @@
     <row r="15" ht="22" customHeight="1">
       <c r="B15" s="32" t="inlineStr">
         <is>
-          <t>Unresearched. No qualitative thesis on file; ranking driven entirely by quantitative signals (see Score decomposition below).</t>
+          <t>Japanese parent Muramoto 80%; ~3.6-4.6% yield; 56% payout; 10yr dividend growth; squeeze-out is upside</t>
         </is>
       </c>
     </row>
@@ -8081,7 +8087,7 @@
         </is>
       </c>
       <c r="C21" s="22" t="n">
-        <v>0.6098453661261224</v>
+        <v>0.7075775903804709</v>
       </c>
       <c r="D21" s="33" t="inlineStr">
         <is>
@@ -8089,7 +8095,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.9079045322105156</v>
+        <v>0.5168569030978339</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -8099,7 +8105,7 @@
         </is>
       </c>
       <c r="C22" s="22" t="n">
-        <v>0.4834847817611555</v>
+        <v>0.6508658603312235</v>
       </c>
       <c r="D22" s="33" t="inlineStr">
         <is>
@@ -8107,7 +8113,7 @@
         </is>
       </c>
       <c r="E22" s="22" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
@@ -8125,7 +8131,7 @@
         </is>
       </c>
       <c r="E23" s="22" t="n">
-        <v>1</v>
+        <v>0.926</v>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
@@ -8135,7 +8141,7 @@
         </is>
       </c>
       <c r="C24" s="22" t="n">
-        <v>0.761567</v>
+        <v>0.7800820000000001</v>
       </c>
       <c r="D24" s="33" t="inlineStr">
         <is>
@@ -8153,7 +8159,7 @@
         </is>
       </c>
       <c r="C25" s="22" t="n">
-        <v>0.4269003334734619</v>
+        <v>0.5225695245785115</v>
       </c>
       <c r="D25" s="33" t="inlineStr">
         <is>
@@ -8161,7 +8167,7 @@
         </is>
       </c>
       <c r="E25" s="34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
@@ -8178,7 +8184,7 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.37188843</v>
+        <v>0.8462543</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
@@ -8186,7 +8192,7 @@
         </is>
       </c>
       <c r="E28" s="23" t="n">
-        <v>104.7508519298697</v>
+        <v>84.50518903603952</v>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
@@ -8196,7 +8202,7 @@
         </is>
       </c>
       <c r="C29" s="22" t="n">
-        <v>0.2541832540201263</v>
+        <v>1.743</v>
       </c>
       <c r="D29" s="33" t="inlineStr">
         <is>
@@ -8204,7 +8210,7 @@
         </is>
       </c>
       <c r="E29" s="22" t="n">
-        <v>-4.049683737461582</v>
+        <v>-1.67116159988576</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
@@ -8224,7 +8230,7 @@
         </is>
       </c>
       <c r="E30" s="23" t="n">
-        <v>13.2643076741945</v>
+        <v>35.31203322577265</v>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
@@ -8234,7 +8240,7 @@
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>5.5</v>
+        <v>5.7241645</v>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
@@ -8242,7 +8248,7 @@
         </is>
       </c>
       <c r="E31" s="23" t="n">
-        <v>30.0813979089536</v>
+        <v>10.96313272568954</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
@@ -8252,7 +8258,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>1.2983886</v>
+        <v>0.3770226</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -8260,7 +8266,7 @@
         </is>
       </c>
       <c r="E32" s="23" t="n">
-        <v>67.661005</v>
+        <v>85.438</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
@@ -8270,7 +8276,7 @@
         </is>
       </c>
       <c r="C33" s="23" t="n">
-        <v>14.81031382345322</v>
+        <v>22.68002247505217</v>
       </c>
       <c r="D33" s="33" t="inlineStr">
         <is>
@@ -8290,7 +8296,7 @@
         </is>
       </c>
       <c r="C34" s="23" t="n">
-        <v>94.09407273683851</v>
+        <v>52.11409371218626</v>
       </c>
       <c r="D34" s="33" t="inlineStr">
         <is>
@@ -8298,7 +8304,7 @@
         </is>
       </c>
       <c r="E34" s="23" t="n">
-        <v>16.08568822862014</v>
+        <v>7.00038199914789</v>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
@@ -8308,7 +8314,7 @@
         </is>
       </c>
       <c r="C35" s="22" t="n">
-        <v>16.75536368504713</v>
+        <v>1.143401385189282</v>
       </c>
       <c r="D35" s="33" t="inlineStr">
         <is>
@@ -8316,7 +8322,7 @@
         </is>
       </c>
       <c r="E35" s="23" t="n">
-        <v>-14.17</v>
+        <v>50.79</v>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1">
@@ -8336,21 +8342,21 @@
     <row r="39" ht="16" customHeight="1">
       <c r="B39" s="35" t="inlineStr">
         <is>
-          <t>·  Sub-book  (P/B 0.37)</t>
+          <t>·  Sub-book  (P/B 0.85)</t>
         </is>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1">
       <c r="B40" s="35" t="inlineStr">
         <is>
-          <t>·  Insider-aligned  (68% insider)</t>
+          <t>·  Insider-aligned  (85% insider)</t>
         </is>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1">
       <c r="B41" s="35" t="inlineStr">
         <is>
-          <t>·  Cluster stack  (4 of 7 inflection signals)</t>
+          <t>·  Cluster stack  (5 of 7 inflection signals)</t>
         </is>
       </c>
     </row>
@@ -8364,7 +8370,7 @@
     <row r="44" ht="18" customHeight="1">
       <c r="B44" s="12" t="inlineStr">
         <is>
-          <t>growth-flip; accelerating sales; under-priced vs fundamentals; cheap+grow (EV/EBIT 0.4x); cash 99% of mcap; cash &gt; EV (16.76x, net cash 94% mcap)</t>
+          <t>growth-flip; first-positive: FCF; accelerating sales; under-priced vs fundamentals; cheap+grow (EV/EBIT 2.0x); cash 55% of mcap; cash &gt; EV (1.14x, net cash 52% mcap)</t>
         </is>
       </c>
     </row>
@@ -8417,7 +8423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -8431,7 +8437,7 @@
     <row r="1" ht="20" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>#22    METCO.BK    Muramoto Electron (Thailand) Public Company Limited</t>
+          <t>#22    KROS    Keros Therapeutics, Inc.</t>
         </is>
       </c>
     </row>
@@ -8449,9 +8455,9 @@
           <t>Verdict</t>
         </is>
       </c>
-      <c r="C3" s="27" t="inlineStr">
-        <is>
-          <t>GREEN</t>
+      <c r="C3" s="37" t="inlineStr">
+        <is>
+          <t>UNRESEARCHED</t>
         </is>
       </c>
       <c r="D3" s="26" t="inlineStr">
@@ -8460,7 +8466,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.095391292032167</v>
+        <v>1.09375163490372</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -8478,7 +8484,7 @@
       </c>
       <c r="B6" s="30" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>US</t>
         </is>
       </c>
     </row>
@@ -8490,7 +8496,7 @@
       </c>
       <c r="B7" s="30" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Health Care</t>
         </is>
       </c>
     </row>
@@ -8502,7 +8508,7 @@
       </c>
       <c r="B8" s="30" t="inlineStr">
         <is>
-          <t>Electronic Equipment, Instruments &amp; Components</t>
+          <t>Biotechnology</t>
         </is>
       </c>
     </row>
@@ -8514,7 +8520,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Small Cap</t>
         </is>
       </c>
     </row>
@@ -8525,7 +8531,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>189173887.7198486</v>
+        <v>224443760</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -8535,7 +8541,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>514626167.5263252</v>
+        <v>244061000</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -8546,7 +8552,7 @@
       </c>
       <c r="B12" s="30" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2025-12-31</t>
         </is>
       </c>
     </row>
@@ -8560,7 +8566,7 @@
     <row r="15" ht="22" customHeight="1">
       <c r="B15" s="32" t="inlineStr">
         <is>
-          <t>Japanese parent Muramoto 80%; ~3.6-4.6% yield; 56% payout; 10yr dividend growth; squeeze-out is upside</t>
+          <t>Unresearched. No qualitative thesis on file; ranking driven entirely by quantitative signals (see Score decomposition below).</t>
         </is>
       </c>
     </row>
@@ -8581,7 +8587,7 @@
         </is>
       </c>
       <c r="C21" s="22" t="n">
-        <v>0.7075775903804709</v>
+        <v>0.6173097965516875</v>
       </c>
       <c r="D21" s="33" t="inlineStr">
         <is>
@@ -8589,7 +8595,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.5168569030978339</v>
+        <v>0.67887376</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -8599,7 +8605,7 @@
         </is>
       </c>
       <c r="C22" s="22" t="n">
-        <v>0.6508658603312235</v>
+        <v>0.5716070773780287</v>
       </c>
       <c r="D22" s="33" t="inlineStr">
         <is>
@@ -8607,7 +8613,7 @@
         </is>
       </c>
       <c r="E22" s="22" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
@@ -8617,7 +8623,7 @@
         </is>
       </c>
       <c r="C23" s="22" t="n">
-        <v>0.7692307692307692</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="D23" s="33" t="inlineStr">
         <is>
@@ -8625,7 +8631,7 @@
         </is>
       </c>
       <c r="E23" s="22" t="n">
-        <v>0.926</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
@@ -8635,7 +8641,7 @@
         </is>
       </c>
       <c r="C24" s="22" t="n">
-        <v>0.7800820000000001</v>
+        <v>0.837901</v>
       </c>
       <c r="D24" s="33" t="inlineStr">
         <is>
@@ -8643,7 +8649,7 @@
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>1.2</v>
+        <v>1.24</v>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
@@ -8653,7 +8659,7 @@
         </is>
       </c>
       <c r="C25" s="22" t="n">
-        <v>0.5225695245785115</v>
+        <v>0.4395225067843441</v>
       </c>
       <c r="D25" s="33" t="inlineStr">
         <is>
@@ -8678,7 +8684,7 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.8462543</v>
+        <v>0.8556312</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
@@ -8686,7 +8692,7 @@
         </is>
       </c>
       <c r="E28" s="23" t="n">
-        <v>84.50518903603952</v>
+        <v>127.0432475398032</v>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
@@ -8696,7 +8702,7 @@
         </is>
       </c>
       <c r="C29" s="22" t="n">
-        <v>1.743</v>
+        <v>0.18</v>
       </c>
       <c r="D29" s="33" t="inlineStr">
         <is>
@@ -8704,7 +8710,7 @@
         </is>
       </c>
       <c r="E29" s="22" t="n">
-        <v>-1.67116159988576</v>
+        <v>-3.916326471524943</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
@@ -8723,8 +8729,10 @@
           <t>ROCE (%)</t>
         </is>
       </c>
-      <c r="E30" s="23" t="n">
-        <v>35.31203322577265</v>
+      <c r="E30" s="25" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
@@ -8733,8 +8741,10 @@
           <t>P/E</t>
         </is>
       </c>
-      <c r="C31" s="22" t="n">
-        <v>5.7241645</v>
+      <c r="C31" s="25" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
@@ -8742,7 +8752,7 @@
         </is>
       </c>
       <c r="E31" s="23" t="n">
-        <v>10.96313272568954</v>
+        <v>28.30357984274423</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
@@ -8752,7 +8762,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.3770226</v>
+        <v>14.948965</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -8760,7 +8770,7 @@
         </is>
       </c>
       <c r="E32" s="23" t="n">
-        <v>85.438</v>
+        <v>3.641</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
@@ -8770,7 +8780,7 @@
         </is>
       </c>
       <c r="C33" s="23" t="n">
-        <v>22.68002247505217</v>
+        <v>36.66783771232035</v>
       </c>
       <c r="D33" s="33" t="inlineStr">
         <is>
@@ -8790,7 +8800,7 @@
         </is>
       </c>
       <c r="C34" s="23" t="n">
-        <v>52.11409371218626</v>
+        <v>135.4560479850007</v>
       </c>
       <c r="D34" s="33" t="inlineStr">
         <is>
@@ -8798,7 +8808,7 @@
         </is>
       </c>
       <c r="E34" s="23" t="n">
-        <v>7.00038199914789</v>
+        <v>6774.957746478873</v>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
@@ -8807,8 +8817,10 @@
           <t>Cash / EV (x)</t>
         </is>
       </c>
-      <c r="C35" s="22" t="n">
-        <v>1.143401385189282</v>
+      <c r="C35" s="25" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="D35" s="33" t="inlineStr">
         <is>
@@ -8816,7 +8828,7 @@
         </is>
       </c>
       <c r="E35" s="23" t="n">
-        <v>50.79</v>
+        <v>-25.62</v>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1">
@@ -8829,79 +8841,71 @@
     <row r="38" ht="16" customHeight="1">
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>·  Cash &gt; EV  (downside floor in place)</t>
+          <t>·  Negative enterprise value</t>
         </is>
       </c>
     </row>
     <row r="39" ht="16" customHeight="1">
       <c r="B39" s="35" t="inlineStr">
         <is>
-          <t>·  Sub-book  (P/B 0.85)</t>
+          <t>·  Sub-book  (P/B 0.86)</t>
         </is>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1">
       <c r="B40" s="35" t="inlineStr">
         <is>
-          <t>·  Insider-aligned  (85% insider)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="16" customHeight="1">
-      <c r="B41" s="35" t="inlineStr">
-        <is>
           <t>·  Cluster stack  (5 of 7 inflection signals)</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="16" customHeight="1">
-      <c r="A43" s="5" t="inlineStr">
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>growth-flip; first-positive: FCF; accelerating sales; under-priced vs fundamentals; cheap+grow (EV/EBIT 2.0x); cash 55% of mcap; cash &gt; EV (1.14x, net cash 52% mcap)</t>
-        </is>
-      </c>
-    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>growth-flip; first-positive: FCF/EBITDA/CFO/NI/ROCE; ROCE improving from &lt;=0; accelerating sales; under-priced vs fundamentals; cash 138% of mcap</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1"/>
     <row r="45" ht="18" customHeight="1"/>
-    <row r="46" ht="18" customHeight="1"/>
+    <row r="48">
+      <c r="A48" s="36" t="n"/>
+      <c r="B48" s="36" t="n"/>
+      <c r="C48" s="36" t="n"/>
+      <c r="D48" s="36" t="n"/>
+      <c r="E48" s="36" t="n"/>
+      <c r="F48" s="36" t="n"/>
+    </row>
     <row r="49">
-      <c r="A49" s="36" t="n"/>
-      <c r="B49" s="36" t="n"/>
-      <c r="C49" s="36" t="n"/>
-      <c r="D49" s="36" t="n"/>
-      <c r="E49" s="36" t="n"/>
-      <c r="F49" s="36" t="n"/>
-    </row>
-    <row r="50">
-      <c r="B50" s="26" t="inlineStr">
+      <c r="B49" s="26" t="inlineStr">
         <is>
           <t>Asymmetry Workbook  ·  Sheet 22 of 50</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="17">
     <mergeCell ref="B40:E40"/>
     <mergeCell ref="B9:E9"/>
-    <mergeCell ref="B41:E41"/>
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="A20:E20"/>
-    <mergeCell ref="A43:E43"/>
     <mergeCell ref="B12:E12"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="B38:E38"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="B43:E45"/>
     <mergeCell ref="B7:E7"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A37:E37"/>
     <mergeCell ref="B39:E39"/>
-    <mergeCell ref="B44:E46"/>
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="B15:E18"/>
     <mergeCell ref="A27:E27"/>
@@ -11564,22 +11568,22 @@
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
-          <t>035610.KQ</t>
+          <t>3798.HK</t>
         </is>
       </c>
       <c r="D18" s="18" t="inlineStr">
         <is>
-          <t>Solborn, Inc.</t>
+          <t>Homeland Interactive Technology Ltd.</t>
         </is>
       </c>
       <c r="E18" s="19" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>CN</t>
         </is>
       </c>
       <c r="F18" s="20" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="G18" s="24" t="inlineStr">
@@ -11588,10 +11592,10 @@
         </is>
       </c>
       <c r="H18" s="22" t="n">
-        <v>1.146648181877715</v>
+        <v>1.146428117925815</v>
       </c>
       <c r="I18" s="22" t="n">
-        <v>0.4404573070670534</v>
+        <v>0.63482887</v>
       </c>
       <c r="J18" s="25" t="inlineStr">
         <is>
@@ -11599,7 +11603,7 @@
         </is>
       </c>
       <c r="K18" s="22" t="n">
-        <v>1.0640486</v>
+        <v>1.2164296</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
@@ -11608,22 +11612,22 @@
       </c>
       <c r="C19" s="17" t="inlineStr">
         <is>
-          <t>3798.HK</t>
+          <t>035610.KQ</t>
         </is>
       </c>
       <c r="D19" s="18" t="inlineStr">
         <is>
-          <t>Homeland Interactive Technology Ltd.</t>
+          <t>Solborn, Inc.</t>
         </is>
       </c>
       <c r="E19" s="19" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="F19" s="20" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="G19" s="24" t="inlineStr">
@@ -11632,10 +11636,10 @@
         </is>
       </c>
       <c r="H19" s="22" t="n">
-        <v>1.146428117925815</v>
+        <v>1.137221610175333</v>
       </c>
       <c r="I19" s="22" t="n">
-        <v>0.63482887</v>
+        <v>0.4404573070670534</v>
       </c>
       <c r="J19" s="25" t="inlineStr">
         <is>
@@ -11643,7 +11647,7 @@
         </is>
       </c>
       <c r="K19" s="22" t="n">
-        <v>1.2164296</v>
+        <v>1.0640486</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
@@ -11736,22 +11740,22 @@
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
-          <t>KROS</t>
+          <t>348350.KQ</t>
         </is>
       </c>
       <c r="D22" s="18" t="inlineStr">
         <is>
-          <t>Keros Therapeutics, Inc.</t>
+          <t>WITHTECH Co., LTD.</t>
         </is>
       </c>
       <c r="E22" s="19" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="F22" s="20" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="G22" s="24" t="inlineStr">
@@ -11760,18 +11764,16 @@
         </is>
       </c>
       <c r="H22" s="22" t="n">
-        <v>1.11727586668782</v>
+        <v>1.113650562417347</v>
       </c>
       <c r="I22" s="22" t="n">
-        <v>0.8556312</v>
-      </c>
-      <c r="J22" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>0.7937623623751395</v>
+      </c>
+      <c r="J22" s="23" t="n">
+        <v>2.8800001</v>
       </c>
       <c r="K22" s="22" t="n">
-        <v>14.948965</v>
+        <v>1.4497193</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
@@ -11780,22 +11782,22 @@
       </c>
       <c r="C23" s="17" t="inlineStr">
         <is>
-          <t>348350.KQ</t>
+          <t>2348.HK</t>
         </is>
       </c>
       <c r="D23" s="18" t="inlineStr">
         <is>
-          <t>WITHTECH Co., LTD.</t>
+          <t>Dawnrays Pharmaceutical (Holdings) Limited</t>
         </is>
       </c>
       <c r="E23" s="19" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>HK</t>
         </is>
       </c>
       <c r="F23" s="20" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="G23" s="24" t="inlineStr">
@@ -11804,16 +11806,16 @@
         </is>
       </c>
       <c r="H23" s="22" t="n">
-        <v>1.113650562417347</v>
+        <v>1.09772165902702</v>
       </c>
       <c r="I23" s="22" t="n">
-        <v>0.7937623623751395</v>
+        <v>0.37188843</v>
       </c>
       <c r="J23" s="23" t="n">
-        <v>2.8800001</v>
+        <v>6.3</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>1.4497193</v>
+        <v>1.2983886</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
@@ -11822,40 +11824,40 @@
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t>2348.HK</t>
+          <t>METCO.BK</t>
         </is>
       </c>
       <c r="D24" s="18" t="inlineStr">
         <is>
-          <t>Dawnrays Pharmaceutical (Holdings) Limited</t>
+          <t>Muramoto Electron (Thailand) Public Company Limited</t>
         </is>
       </c>
       <c r="E24" s="19" t="inlineStr">
         <is>
-          <t>HK</t>
+          <t>TH</t>
         </is>
       </c>
       <c r="F24" s="20" t="inlineStr">
         <is>
-          <t>Health Care</t>
-        </is>
-      </c>
-      <c r="G24" s="24" t="inlineStr">
-        <is>
-          <t>UNRESEARCHED</t>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="G24" s="21" t="inlineStr">
+        <is>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="H24" s="22" t="n">
-        <v>1.09772165902702</v>
+        <v>1.095391292032167</v>
       </c>
       <c r="I24" s="22" t="n">
-        <v>0.37188843</v>
+        <v>0.8462543</v>
       </c>
       <c r="J24" s="23" t="n">
-        <v>6.3</v>
+        <v>10.24</v>
       </c>
       <c r="K24" s="22" t="n">
-        <v>1.2983886</v>
+        <v>0.3770226</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
@@ -11864,40 +11866,42 @@
       </c>
       <c r="C25" s="17" t="inlineStr">
         <is>
-          <t>METCO.BK</t>
+          <t>KROS</t>
         </is>
       </c>
       <c r="D25" s="18" t="inlineStr">
         <is>
-          <t>Muramoto Electron (Thailand) Public Company Limited</t>
+          <t>Keros Therapeutics, Inc.</t>
         </is>
       </c>
       <c r="E25" s="19" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>US</t>
         </is>
       </c>
       <c r="F25" s="20" t="inlineStr">
         <is>
-          <t>Information Technology</t>
-        </is>
-      </c>
-      <c r="G25" s="21" t="inlineStr">
-        <is>
-          <t>GREEN</t>
+          <t>Health Care</t>
+        </is>
+      </c>
+      <c r="G25" s="24" t="inlineStr">
+        <is>
+          <t>UNRESEARCHED</t>
         </is>
       </c>
       <c r="H25" s="22" t="n">
-        <v>1.095391292032167</v>
+        <v>1.09375163490372</v>
       </c>
       <c r="I25" s="22" t="n">
-        <v>0.8462543</v>
-      </c>
-      <c r="J25" s="23" t="n">
-        <v>10.24</v>
+        <v>0.8556312</v>
+      </c>
+      <c r="J25" s="25" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="K25" s="22" t="n">
-        <v>0.3770226</v>
+        <v>14.948965</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">

</xml_diff>

<commit_message>
Full render: all 20 books de-ghosted (real UMBF restored, 213 ghosts removed)
Regenerated on the de-ghosted data — wrong-price duplicate lines (UMBFO etc.)
no longer rank or display corrupt ratios; the real primary listings are back.
87 archetypes; audit 109 checks, 0 FAIL, 0 WARN; mutation 32/32.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/asymmetry_harvard_workbook.xlsx
+++ b/asymmetry_harvard_workbook.xlsx
@@ -26188,16 +26188,16 @@
         <v>1</v>
       </c>
       <c r="E14" s="34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F14" s="34" t="n">
         <v>0</v>
       </c>
       <c r="G14" s="34" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H14" s="23" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
Rebuild all books on merged D&A/financing coverage
Regenerated the render-managed workbooks (and NMS candidates) on the master
with the Yahoo statement gap-fill applied (da_ttm 25,592 / capex_ttm 26,148 /
financing_cf_ttm 11,971), so the D&A/capex-dependent columns and archetypes
reflect the extended, non-US coverage.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/asymmetry_harvard_workbook.xlsx
+++ b/asymmetry_harvard_workbook.xlsx
@@ -55,9 +55,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="43_4625_T" sheetId="46" state="visible" r:id="rId46"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="44_1V5_F" sheetId="47" state="visible" r:id="rId47"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="45_CAAS" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="46_0725_HK" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="46_1281_HK" sheetId="49" state="visible" r:id="rId49"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="47_131090_KQ" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="48_1281_HK" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="48_0725_HK" sheetId="51" state="visible" r:id="rId51"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="49_052790_KQ" sheetId="52" state="visible" r:id="rId52"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50_3954_T" sheetId="53" state="visible" r:id="rId53"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="54" state="visible" r:id="rId54"/>
@@ -756,7 +756,7 @@
     <row r="11" ht="24" customHeight="1">
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>26,385</t>
+          <t>26,389</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>25,984</t>
+          <t>25,988</t>
         </is>
       </c>
     </row>
@@ -835,7 +835,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>This workbook documents the top 50 names from a global universe of 26,385 equities ranked by an entry-today asymmetry score. The upside leg weights factors Anna Yartseva (CAFE WP 33, 2025) finds predictive of 10-bagger outcomes — FCF yield, book-to-market, small size, profitability level, asset-growth gate, contra-momentum. The downside floor leg combines Graham net-net, cash &gt; EV, sub-book and negative-EV signals. Each candidate has been qualitatively reviewed and assigned a verdict of GREEN (high-conviction), YELLOW (risk-flagged), RED (avoid) or UNRESEARCHED. Sheets sequence as Cover, Methodology, Index, per-name pages, Coverage, References.</t>
+          <t>This workbook documents the top 50 names from a global universe of 26,389 equities ranked by an entry-today asymmetry score. The upside leg weights factors Anna Yartseva (CAFE WP 33, 2025) finds predictive of 10-bagger outcomes — FCF yield, book-to-market, small size, profitability level, asset-growth gate, contra-momentum. The downside floor leg combines Graham net-net, cash &gt; EV, sub-book and negative-EV signals. Each candidate has been qualitatively reviewed and assigned a verdict of GREEN (high-conviction), YELLOW (risk-flagged), RED (avoid) or UNRESEARCHED. Sheets sequence as Cover, Methodology, Index, per-name pages, Coverage, References.</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.173223187173692</v>
+        <v>1.172504383176419</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>77653786.95794658</v>
+        <v>78237641.18890361</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -1051,7 +1051,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.725824299626438</v>
+        <v>0.7249200996264381</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -1140,7 +1140,7 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.601293</v>
+        <v>0.605814</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
@@ -1194,7 +1194,7 @@
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>10.23077</v>
+        <v>10.307693</v>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.5709076</v>
+        <v>0.5752</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -1296,7 +1296,7 @@
     <row r="39" ht="16" customHeight="1">
       <c r="B39" s="35" t="inlineStr">
         <is>
-          <t>·  Sub-book  (P/B 0.60)</t>
+          <t>·  Sub-book  (P/B 0.61)</t>
         </is>
       </c>
     </row>
@@ -2951,7 +2951,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>97649721.25524984</v>
+        <v>97745653.94004904</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -3176,7 +3176,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>1.225791</v>
+        <v>1.2269952</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -3439,7 +3439,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>69110133.31576708</v>
+        <v>69063217.17478731</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -3933,7 +3933,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>98540142.03049168</v>
+        <v>98798555.87781604</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -4158,7 +4158,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.3509070426787583</v>
+        <v>0.3518272690665361</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -5413,7 +5413,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>18429222.51684681</v>
+        <v>18347168.83320943</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -5638,7 +5638,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.20313144</v>
+        <v>0.20222703</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -6982,7 +6982,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.099278313855842</v>
+        <v>1.101049539651115</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -7047,7 +7047,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>50773986.45186899</v>
+        <v>48701579.34159086</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -7111,7 +7111,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.6370614891453174</v>
+        <v>0.6392964091453174</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -7200,7 +7200,7 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.2737778</v>
+        <v>0.2626032</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
@@ -7220,7 +7220,7 @@
         </is>
       </c>
       <c r="C29" s="22" t="n">
-        <v>-4.083374947411143</v>
+        <v>-4.345596984910629</v>
       </c>
       <c r="D29" s="33" t="inlineStr">
         <is>
@@ -7238,7 +7238,7 @@
         </is>
       </c>
       <c r="C30" s="22" t="n">
-        <v>-2.817688644880061</v>
+        <v>-2.998632121052401</v>
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
@@ -7256,7 +7256,7 @@
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>16.98113681911677</v>
+        <v>16.28802936107025</v>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
@@ -7274,7 +7274,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>1.200266309500878</v>
+        <v>1.151275859708347</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -7358,7 +7358,7 @@
     <row r="39" ht="16" customHeight="1">
       <c r="B39" s="35" t="inlineStr">
         <is>
-          <t>·  Sub-book  (P/B 0.27)</t>
+          <t>·  Sub-book  (P/B 0.26)</t>
         </is>
       </c>
     </row>
@@ -8027,7 +8027,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>72336165.70478408</v>
+        <v>71024071.39044254</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -8091,7 +8091,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.762087879864858</v>
+        <v>0.764433611864858</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -8180,7 +8180,7 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.6466033</v>
+        <v>0.63487464</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
@@ -8236,7 +8236,7 @@
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>8.007805236580204</v>
+        <v>7.862552918892367</v>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
@@ -8254,7 +8254,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.3068591</v>
+        <v>0.30129302</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -8338,7 +8338,7 @@
     <row r="39" ht="16" customHeight="1">
       <c r="B39" s="35" t="inlineStr">
         <is>
-          <t>·  Sub-book  (P/B 0.65)</t>
+          <t>·  Sub-book  (P/B 0.63)</t>
         </is>
       </c>
     </row>
@@ -8525,7 +8525,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>23924676.0523474</v>
+        <v>24329555.49054453</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -8750,7 +8750,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>1.858148</v>
+        <v>1.8895935</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -8942,7 +8942,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.095466595284029</v>
+        <v>1.094907872286137</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -9007,7 +9007,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>184192477.3257772</v>
+        <v>185001225.2794639</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -9071,7 +9071,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.670534450302693</v>
+        <v>0.669809932302693</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -9160,7 +9160,7 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.82505226</v>
+        <v>0.82867485</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
@@ -9214,7 +9214,7 @@
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>61.84160092575997</v>
+        <v>62.11313355796926</v>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
@@ -9232,7 +9232,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.45700946</v>
+        <v>0.45901608</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -9440,7 +9440,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.092825899825435</v>
+        <v>1.092706777931071</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -9505,7 +9505,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>37283078.28963859</v>
+        <v>37332395.30343874</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -9569,7 +9569,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.6290377506939995</v>
+        <v>0.6288874306939994</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -9658,7 +9658,7 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.5681878</v>
+        <v>0.5689394</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
@@ -9712,7 +9712,7 @@
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>260.1177048004683</v>
+        <v>260.4617812293953</v>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
@@ -9730,7 +9730,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.9468284</v>
+        <v>0.9480809</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -9887,7 +9887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -9930,7 +9930,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.084630529981028</v>
+        <v>1.082675977629569</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -9993,7 +9993,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>20660894.65984212</v>
+        <v>21714424.70673309</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -10057,7 +10057,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.6837826681597364</v>
+        <v>0.6811989281597365</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -10146,7 +10146,7 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.9870813000000001</v>
+        <v>1.0374141</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
@@ -10202,7 +10202,7 @@
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>17.57093</v>
+        <v>18.476095</v>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
@@ -10220,7 +10220,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>2.8326097</v>
+        <v>2.9770486</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -10304,72 +10304,64 @@
     <row r="39" ht="16" customHeight="1">
       <c r="B39" s="35" t="inlineStr">
         <is>
-          <t>·  Sub-book  (P/B 0.99)</t>
+          <t>·  Insider-aligned  (67% insider)</t>
         </is>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1">
       <c r="B40" s="35" t="inlineStr">
         <is>
-          <t>·  Insider-aligned  (67% insider)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="16" customHeight="1">
-      <c r="B41" s="35" t="inlineStr">
-        <is>
           <t>·  Cluster stack  (5 of 7 inflection signals)</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="16" customHeight="1">
-      <c r="A43" s="5" t="inlineStr">
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="B44" s="12" t="inlineStr">
+    <row r="43" ht="18" customHeight="1">
+      <c r="B43" s="12" t="inlineStr">
         <is>
           <t>growth-flip; first-positive: FCF; accelerating sales; under-priced vs fundamentals; cheap+grow (EV/EBIT 1.0x); cash 93% of mcap; cash &gt; EV (9.08x, net cash 91% mcap)</t>
         </is>
       </c>
     </row>
+    <row r="44" ht="18" customHeight="1"/>
     <row r="45" ht="18" customHeight="1"/>
-    <row r="46" ht="18" customHeight="1"/>
+    <row r="48">
+      <c r="A48" s="36" t="n"/>
+      <c r="B48" s="36" t="n"/>
+      <c r="C48" s="36" t="n"/>
+      <c r="D48" s="36" t="n"/>
+      <c r="E48" s="36" t="n"/>
+      <c r="F48" s="36" t="n"/>
+    </row>
     <row r="49">
-      <c r="A49" s="36" t="n"/>
-      <c r="B49" s="36" t="n"/>
-      <c r="C49" s="36" t="n"/>
-      <c r="D49" s="36" t="n"/>
-      <c r="E49" s="36" t="n"/>
-      <c r="F49" s="36" t="n"/>
-    </row>
-    <row r="50">
-      <c r="B50" s="26" t="inlineStr">
+      <c r="B49" s="26" t="inlineStr">
         <is>
           <t>Asymmetry Workbook  ·  Sheet 25 of 50</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="17">
     <mergeCell ref="B40:E40"/>
     <mergeCell ref="B9:E9"/>
-    <mergeCell ref="B41:E41"/>
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="A20:E20"/>
-    <mergeCell ref="A43:E43"/>
     <mergeCell ref="B12:E12"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="B38:E38"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="B43:E45"/>
     <mergeCell ref="B7:E7"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A37:E37"/>
     <mergeCell ref="B39:E39"/>
-    <mergeCell ref="B44:E46"/>
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="B15:E18"/>
     <mergeCell ref="A27:E27"/>
@@ -11001,7 +10993,7 @@
         <v>2.42</v>
       </c>
       <c r="K4" s="22" t="n">
-        <v>0.19837561</v>
+        <v>0.19885361</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
@@ -11160,10 +11152,10 @@
         </is>
       </c>
       <c r="H8" s="22" t="n">
-        <v>1.214607294531874</v>
+        <v>1.213706119342358</v>
       </c>
       <c r="I8" s="22" t="n">
-        <v>0.64328694</v>
+        <v>0.64855975</v>
       </c>
       <c r="J8" s="25" t="inlineStr">
         <is>
@@ -11171,7 +11163,7 @@
         </is>
       </c>
       <c r="K8" s="22" t="n">
-        <v>1.06764828969794</v>
+        <v>1.076399494270387</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
@@ -11213,7 +11205,7 @@
         <v>2.77</v>
       </c>
       <c r="K9" s="22" t="n">
-        <v>0.47688493</v>
+        <v>0.47579452</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
@@ -11246,16 +11238,16 @@
         </is>
       </c>
       <c r="H10" s="22" t="n">
-        <v>1.173223187173692</v>
+        <v>1.172504383176419</v>
       </c>
       <c r="I10" s="22" t="n">
-        <v>0.601293</v>
+        <v>0.605814</v>
       </c>
       <c r="J10" s="23" t="n">
         <v>4.21</v>
       </c>
       <c r="K10" s="22" t="n">
-        <v>0.5709076</v>
+        <v>0.5752</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
@@ -11423,7 +11415,7 @@
         <v>4.9200002</v>
       </c>
       <c r="K14" s="22" t="n">
-        <v>1.225791</v>
+        <v>1.2269952</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -11509,7 +11501,7 @@
         <v>2.79</v>
       </c>
       <c r="K16" s="22" t="n">
-        <v>0.3509070426787583</v>
+        <v>0.3518272690665361</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
@@ -11637,7 +11629,7 @@
         <v>2.0299999</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>0.20313144</v>
+        <v>0.20222703</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
@@ -11756,10 +11748,10 @@
         </is>
       </c>
       <c r="H22" s="22" t="n">
-        <v>1.099278313855842</v>
+        <v>1.101049539651115</v>
       </c>
       <c r="I22" s="22" t="n">
-        <v>0.2737778</v>
+        <v>0.2626032</v>
       </c>
       <c r="J22" s="25" t="inlineStr">
         <is>
@@ -11767,7 +11759,7 @@
         </is>
       </c>
       <c r="K22" s="22" t="n">
-        <v>1.200266309500878</v>
+        <v>1.151275859708347</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
@@ -11845,13 +11837,13 @@
         <v>1.097238104899035</v>
       </c>
       <c r="I24" s="22" t="n">
-        <v>0.6466033</v>
+        <v>0.63487464</v>
       </c>
       <c r="J24" s="23" t="n">
         <v>2.4300002</v>
       </c>
       <c r="K24" s="22" t="n">
-        <v>0.3068591</v>
+        <v>0.30129302</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
@@ -11895,7 +11887,7 @@
         </is>
       </c>
       <c r="K25" s="22" t="n">
-        <v>1.858148</v>
+        <v>1.8895935</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
@@ -11928,16 +11920,16 @@
         </is>
       </c>
       <c r="H26" s="22" t="n">
-        <v>1.095466595284029</v>
+        <v>1.094907872286137</v>
       </c>
       <c r="I26" s="22" t="n">
-        <v>0.82505226</v>
+        <v>0.82867485</v>
       </c>
       <c r="J26" s="23" t="n">
         <v>3.55</v>
       </c>
       <c r="K26" s="22" t="n">
-        <v>0.45700946</v>
+        <v>0.45901608</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
@@ -11970,10 +11962,10 @@
         </is>
       </c>
       <c r="H27" s="22" t="n">
-        <v>1.092825899825435</v>
+        <v>1.092706777931071</v>
       </c>
       <c r="I27" s="22" t="n">
-        <v>0.5681878</v>
+        <v>0.5689394</v>
       </c>
       <c r="J27" s="25" t="inlineStr">
         <is>
@@ -11981,7 +11973,7 @@
         </is>
       </c>
       <c r="K27" s="22" t="n">
-        <v>0.9468284</v>
+        <v>0.9480809</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
@@ -12014,16 +12006,16 @@
         </is>
       </c>
       <c r="H28" s="22" t="n">
-        <v>1.084630529981028</v>
+        <v>1.082675977629569</v>
       </c>
       <c r="I28" s="22" t="n">
-        <v>0.9870813000000001</v>
+        <v>1.0374141</v>
       </c>
       <c r="J28" s="23" t="n">
         <v>0.5599999999999999</v>
       </c>
       <c r="K28" s="22" t="n">
-        <v>2.8326097</v>
+        <v>2.9770486</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
@@ -12151,7 +12143,7 @@
         <v>5.71</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>0.5645629</v>
+        <v>0.5612516400000001</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
@@ -12182,16 +12174,16 @@
         </is>
       </c>
       <c r="H32" s="22" t="n">
-        <v>1.073817836048235</v>
+        <v>1.072794052555671</v>
       </c>
       <c r="I32" s="22" t="n">
-        <v>0.5712140999999999</v>
+        <v>0.57788193</v>
       </c>
       <c r="J32" s="23" t="n">
         <v>1.39</v>
       </c>
       <c r="K32" s="22" t="n">
-        <v>0.5015371</v>
+        <v>0.50739163</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
@@ -12233,7 +12225,7 @@
         <v>2.8800001</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>1.4025122</v>
+        <v>1.4009893</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
@@ -12264,16 +12256,16 @@
         </is>
       </c>
       <c r="H34" s="22" t="n">
-        <v>1.069061043495279</v>
+        <v>1.068682304326143</v>
       </c>
       <c r="I34" s="22" t="n">
-        <v>0.60156065</v>
+        <v>0.6041536</v>
       </c>
       <c r="J34" s="23" t="n">
         <v>1.23000005</v>
       </c>
       <c r="K34" s="22" t="n">
-        <v>0.44866917</v>
+        <v>0.45060313</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
@@ -12309,13 +12301,13 @@
         <v>1.066842547335759</v>
       </c>
       <c r="I35" s="22" t="n">
-        <v>0.6536218499999999</v>
+        <v>0.6513203400000001</v>
       </c>
       <c r="J35" s="23" t="n">
         <v>1.07</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>2.4318655</v>
+        <v>2.4233024</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
@@ -12401,7 +12393,7 @@
         </is>
       </c>
       <c r="K37" s="22" t="n">
-        <v>0.23204216</v>
+        <v>0.23250532</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
@@ -12432,16 +12424,16 @@
         </is>
       </c>
       <c r="H38" s="22" t="n">
-        <v>1.058431562072892</v>
+        <v>1.060366004632101</v>
       </c>
       <c r="I38" s="22" t="n">
-        <v>0.8213800999999999</v>
+        <v>0.809476</v>
       </c>
       <c r="J38" s="23" t="n">
         <v>4.9200002</v>
       </c>
       <c r="K38" s="22" t="n">
-        <v>2.000695</v>
+        <v>1.9716996</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
@@ -12474,16 +12466,16 @@
         </is>
       </c>
       <c r="H39" s="22" t="n">
-        <v>1.052608565093393</v>
+        <v>1.052813435988574</v>
       </c>
       <c r="I39" s="22" t="n">
-        <v>0.830867</v>
+        <v>0.8297809</v>
       </c>
       <c r="J39" s="23" t="n">
         <v>5.35</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>0.7343785</v>
+        <v>0.7334186</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
@@ -12770,16 +12762,16 @@
         </is>
       </c>
       <c r="H46" s="22" t="n">
-        <v>1.027618535300892</v>
+        <v>1.027683931197308</v>
       </c>
       <c r="I46" s="22" t="n">
-        <v>0.40647167</v>
+        <v>0.40600014</v>
       </c>
       <c r="J46" s="23" t="n">
         <v>2.77</v>
       </c>
       <c r="K46" s="22" t="n">
-        <v>0.34490073</v>
+        <v>0.3445006</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
@@ -12856,10 +12848,10 @@
         </is>
       </c>
       <c r="H48" s="22" t="n">
-        <v>1.026328294118021</v>
+        <v>1.026123465125633</v>
       </c>
       <c r="I48" s="22" t="n">
-        <v>0.3576042</v>
+        <v>0.35896394</v>
       </c>
       <c r="J48" s="25" t="inlineStr">
         <is>
@@ -12867,7 +12859,7 @@
         </is>
       </c>
       <c r="K48" s="22" t="n">
-        <v>0.19008878</v>
+        <v>0.19081154</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
@@ -12876,12 +12868,12 @@
       </c>
       <c r="C49" s="17" t="inlineStr">
         <is>
-          <t>0725.HK</t>
+          <t>1281.HK</t>
         </is>
       </c>
       <c r="D49" s="18" t="inlineStr">
         <is>
-          <t>Perennial International Limited</t>
+          <t>LongiTech Smart Energy Holding Limited</t>
         </is>
       </c>
       <c r="E49" s="19" t="inlineStr">
@@ -12891,25 +12883,27 @@
       </c>
       <c r="F49" s="20" t="inlineStr">
         <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="G49" s="21" t="inlineStr">
-        <is>
-          <t>GREEN</t>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="G49" s="24" t="inlineStr">
+        <is>
+          <t>UNRESEARCHED</t>
         </is>
       </c>
       <c r="H49" s="22" t="n">
-        <v>1.019908786675609</v>
+        <v>1.024547950517395</v>
       </c>
       <c r="I49" s="22" t="n">
-        <v>0.40812057</v>
-      </c>
-      <c r="J49" s="23" t="n">
-        <v>9</v>
+        <v>0.14083</v>
+      </c>
+      <c r="J49" s="25" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="K49" s="22" t="n">
-        <v>0.47891504</v>
+        <v>0.9045904154520544</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
@@ -12951,7 +12945,7 @@
         <v>4.3</v>
       </c>
       <c r="K50" s="22" t="n">
-        <v>2.2538886</v>
+        <v>2.2647114</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
@@ -12960,12 +12954,12 @@
       </c>
       <c r="C51" s="17" t="inlineStr">
         <is>
-          <t>1281.HK</t>
+          <t>0725.HK</t>
         </is>
       </c>
       <c r="D51" s="18" t="inlineStr">
         <is>
-          <t>LongiTech Smart Energy Holding Limited</t>
+          <t>Perennial International Limited</t>
         </is>
       </c>
       <c r="E51" s="19" t="inlineStr">
@@ -12975,27 +12969,25 @@
       </c>
       <c r="F51" s="20" t="inlineStr">
         <is>
-          <t>Utilities</t>
-        </is>
-      </c>
-      <c r="G51" s="24" t="inlineStr">
-        <is>
-          <t>UNRESEARCHED</t>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="G51" s="21" t="inlineStr">
+        <is>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="H51" s="22" t="n">
-        <v>1.016413963344826</v>
+        <v>1.019209861728622</v>
       </c>
       <c r="I51" s="22" t="n">
-        <v>0.13929923</v>
-      </c>
-      <c r="J51" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>0.41230643</v>
+      </c>
+      <c r="J51" s="23" t="n">
+        <v>9</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>0.8947578844443459</v>
+        <v>0.483827</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
@@ -13039,7 +13031,7 @@
         </is>
       </c>
       <c r="K52" s="22" t="n">
-        <v>0.6022702</v>
+        <v>0.6088967</v>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
@@ -13257,7 +13249,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>227119088.1089789</v>
+        <v>229039477.8522077</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -13735,7 +13727,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>24146193.53754446</v>
+        <v>24004571.73281214</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -13960,7 +13952,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.5645629</v>
+        <v>0.5612516400000001</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -14168,7 +14160,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.073817836048235</v>
+        <v>1.072794052555671</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -14229,7 +14221,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>56815040.56741953</v>
+        <v>57478251.0455513</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -14293,7 +14285,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.6487400331688689</v>
+        <v>0.6474064671688688</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -14382,7 +14374,7 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.5712140999999999</v>
+        <v>0.57788193</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
@@ -14456,7 +14448,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.5015371</v>
+        <v>0.50739163</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -14540,7 +14532,7 @@
     <row r="39" ht="16" customHeight="1">
       <c r="B39" s="35" t="inlineStr">
         <is>
-          <t>·  Sub-book  (P/B 0.57)</t>
+          <t>·  Sub-book  (P/B 0.58)</t>
         </is>
       </c>
     </row>
@@ -14727,7 +14719,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>58876338.41682063</v>
+        <v>58812410.08447371</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -14954,7 +14946,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>1.4025122</v>
+        <v>1.4009893</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -15154,7 +15146,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.069061043495279</v>
+        <v>1.068682304326143</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -15215,7 +15207,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>23665919.52022672</v>
+        <v>23767929.1761291</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -15279,7 +15271,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.7138157648456206</v>
+        <v>0.7132971748456206</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -15368,7 +15360,7 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.60156065</v>
+        <v>0.6041536</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
@@ -15424,7 +15416,7 @@
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>6.309491</v>
+        <v>6.3366876</v>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
@@ -15442,7 +15434,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.44866917</v>
+        <v>0.45060313</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -15713,7 +15705,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>13364747.41860322</v>
+        <v>13317687.95425586</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -15777,7 +15769,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.7989604609929413</v>
+        <v>0.7994207629929412</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -15866,7 +15858,7 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.6536218499999999</v>
+        <v>0.6513203400000001</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
@@ -15922,7 +15914,7 @@
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>19.346048</v>
+        <v>19.27793</v>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
@@ -15940,7 +15932,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>2.4318655</v>
+        <v>2.4233024</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -16695,7 +16687,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>88338287.18595138</v>
+        <v>88514613.86107269</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -16922,7 +16914,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.23204216</v>
+        <v>0.23250532</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -17114,7 +17106,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.058431562072892</v>
+        <v>1.060366004632101</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -17175,7 +17167,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>646742342.4944687</v>
+        <v>637369300.1551437</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -17239,7 +17231,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.5526672824261241</v>
+        <v>0.555048102426124</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -17328,7 +17320,7 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.8213800999999999</v>
+        <v>0.809476</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
@@ -17382,7 +17374,7 @@
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>5.693821</v>
+        <v>5.611302</v>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
@@ -17400,7 +17392,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>2.000695</v>
+        <v>1.9716996</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -17484,7 +17476,7 @@
     <row r="39" ht="16" customHeight="1">
       <c r="B39" s="35" t="inlineStr">
         <is>
-          <t>·  Sub-book  (P/B 0.82)</t>
+          <t>·  Sub-book  (P/B 0.81)</t>
         </is>
       </c>
     </row>
@@ -17600,7 +17592,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.052608565093393</v>
+        <v>1.052813435988574</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -17665,7 +17657,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>64263095.03524991</v>
+        <v>64179093.31776353</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -17729,7 +17721,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.3660571749715599</v>
+        <v>0.3662743949715599</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -17818,7 +17810,7 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.830867</v>
+        <v>0.8297809</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
@@ -17872,7 +17864,7 @@
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>6.8931336</v>
+        <v>6.884123</v>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
@@ -17890,7 +17882,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.7343785</v>
+        <v>0.7334186</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -18161,7 +18153,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>34909646.27042425</v>
+        <v>34993764.18925035</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -18386,7 +18378,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.19837561</v>
+        <v>0.19885361</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -21111,7 +21103,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>64731618.55333321</v>
+        <v>64845983.34468452</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -21536,7 +21528,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.027618535300892</v>
+        <v>1.027683931197308</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -21601,7 +21593,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>28617906.59480798</v>
+        <v>28584706.18959533</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -21665,7 +21657,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.7319063412389546</v>
+        <v>0.7320006472389546</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -21754,7 +21746,7 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.40647167</v>
+        <v>0.40600014</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
@@ -21808,7 +21800,7 @@
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>4.8549705</v>
+        <v>4.849338</v>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
@@ -21826,7 +21818,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.34490073</v>
+        <v>0.3445006</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -22522,7 +22514,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.026328294118021</v>
+        <v>1.026123465125633</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -22587,7 +22579,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>158697904</v>
+        <v>159301312</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -22651,7 +22643,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.6126387733251275</v>
+        <v>0.6123668253251274</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -22740,7 +22732,7 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.3576042</v>
+        <v>0.35896394</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
@@ -22794,7 +22786,7 @@
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>2.7684212</v>
+        <v>2.7789476</v>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
@@ -22812,7 +22804,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.19008878</v>
+        <v>0.19081154</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -22951,7 +22943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -22965,7 +22957,7 @@
     <row r="1" ht="20" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>#46    0725.HK    Perennial International Limited</t>
+          <t>#46    1281.HK    LongiTech Smart Energy Holding Limited</t>
         </is>
       </c>
     </row>
@@ -22983,9 +22975,9 @@
           <t>Verdict</t>
         </is>
       </c>
-      <c r="C3" s="27" t="inlineStr">
-        <is>
-          <t>GREEN</t>
+      <c r="C3" s="37" t="inlineStr">
+        <is>
+          <t>UNRESEARCHED</t>
         </is>
       </c>
       <c r="D3" s="26" t="inlineStr">
@@ -22994,7 +22986,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.019908786675609</v>
+        <v>1.024547950517395</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -23024,7 +23016,7 @@
       </c>
       <c r="B7" s="30" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Utilities</t>
         </is>
       </c>
     </row>
@@ -23036,7 +23028,7 @@
       </c>
       <c r="B8" s="30" t="inlineStr">
         <is>
-          <t>Electrical Equipment</t>
+          <t>Independent Power and Renewable Electricity Producers</t>
         </is>
       </c>
     </row>
@@ -23059,7 +23051,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>24753283.59752344</v>
+        <v>17428710.39306092</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -23069,7 +23061,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>50498298.96777866</v>
+        <v>19266963.3630279</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -23080,7 +23072,7 @@
       </c>
       <c r="B12" s="30" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>–</t>
         </is>
       </c>
     </row>
@@ -23094,7 +23086,7 @@
     <row r="15" ht="22" customHeight="1">
       <c r="B15" s="32" t="inlineStr">
         <is>
-          <t>Perennial International - electric cable family business; ~6% TTM dividend yield with intact payouts; P/B 0.46</t>
+          <t>Unresearched. No qualitative thesis on file; ranking driven entirely by quantitative signals (see Score decomposition below).</t>
         </is>
       </c>
     </row>
@@ -23115,7 +23107,7 @@
         </is>
       </c>
       <c r="C21" s="22" t="n">
-        <v>0.6381708462961632</v>
+        <v>0.6291497860677019</v>
       </c>
       <c r="D21" s="33" t="inlineStr">
         <is>
@@ -23123,7 +23115,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.4716463047139654</v>
+        <v>0.6626164776618847</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -23133,7 +23125,7 @@
         </is>
       </c>
       <c r="C22" s="22" t="n">
-        <v>0.5294406377810695</v>
+        <v>0.5145782893017455</v>
       </c>
       <c r="D22" s="33" t="inlineStr">
         <is>
@@ -23141,7 +23133,7 @@
         </is>
       </c>
       <c r="E22" s="22" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
@@ -23159,7 +23151,7 @@
         </is>
       </c>
       <c r="E23" s="22" t="n">
-        <v>0.991</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
@@ -23169,7 +23161,7 @@
         </is>
       </c>
       <c r="C24" s="22" t="n">
-        <v>0.820348</v>
+        <v>0.8794749681014746</v>
       </c>
       <c r="D24" s="33" t="inlineStr">
         <is>
@@ -23177,7 +23169,7 @@
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>1.2</v>
+        <v>1.1528</v>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
@@ -23187,7 +23179,7 @@
         </is>
       </c>
       <c r="C25" s="22" t="n">
-        <v>0.5524636352202518</v>
+        <v>0.4655292998699878</v>
       </c>
       <c r="D25" s="33" t="inlineStr">
         <is>
@@ -23195,7 +23187,7 @@
         </is>
       </c>
       <c r="E25" s="34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
@@ -23212,15 +23204,17 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.40812057</v>
+        <v>0.14083</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
           <t>NCAV / mcap (%)</t>
         </is>
       </c>
-      <c r="E28" s="23" t="n">
-        <v>119.585308118896</v>
+      <c r="E28" s="25" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
@@ -23230,7 +23224,7 @@
         </is>
       </c>
       <c r="C29" s="22" t="n">
-        <v>1.985515932474278</v>
+        <v>-3.322634386904862</v>
       </c>
       <c r="D29" s="33" t="inlineStr">
         <is>
@@ -23238,7 +23232,7 @@
         </is>
       </c>
       <c r="E29" s="22" t="n">
-        <v>-2.129477574667865</v>
+        <v>-7.396120066301267</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
@@ -23258,7 +23252,7 @@
         </is>
       </c>
       <c r="E30" s="23" t="n">
-        <v>11.90882409257052</v>
+        <v>2.15667527759927</v>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
@@ -23268,7 +23262,7 @@
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>6.5</v>
+        <v>7.585980566515093</v>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
@@ -23276,7 +23270,7 @@
         </is>
       </c>
       <c r="E31" s="23" t="n">
-        <v>12.64845605700712</v>
+        <v>31.31714285714285</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
@@ -23286,7 +23280,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.47891504</v>
+        <v>0.9045904154520544</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -23294,7 +23288,7 @@
         </is>
       </c>
       <c r="E32" s="23" t="n">
-        <v>74.361</v>
+        <v>65.373003</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
@@ -23304,7 +23298,7 @@
         </is>
       </c>
       <c r="C33" s="23" t="n">
-        <v>24.22527118078666</v>
+        <v>99.15826792971392</v>
       </c>
       <c r="D33" s="33" t="inlineStr">
         <is>
@@ -23324,7 +23318,7 @@
         </is>
       </c>
       <c r="C34" s="23" t="n">
-        <v>50.5420998322809</v>
+        <v>181.9727797636792</v>
       </c>
       <c r="D34" s="33" t="inlineStr">
         <is>
@@ -23332,7 +23326,7 @@
         </is>
       </c>
       <c r="E34" s="23" t="n">
-        <v>20.44019989165434</v>
+        <v>22.5586749656398</v>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
@@ -23342,7 +23336,7 @@
         </is>
       </c>
       <c r="C35" s="22" t="n">
-        <v>1.021921589561637</v>
+        <v>1.54376636882513</v>
       </c>
       <c r="D35" s="33" t="inlineStr">
         <is>
@@ -23350,7 +23344,7 @@
         </is>
       </c>
       <c r="E35" s="23" t="n">
-        <v>32.5</v>
+        <v>-24.14</v>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1">
@@ -23370,60 +23364,50 @@
     <row r="39" ht="16" customHeight="1">
       <c r="B39" s="35" t="inlineStr">
         <is>
-          <t>·  Sub-book  (P/B 0.41)</t>
+          <t>·  Sub-book  (P/B 0.14)</t>
         </is>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1">
       <c r="B40" s="35" t="inlineStr">
         <is>
-          <t>·  Insider-aligned  (74% insider)</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>NOTES</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>growth-flip; accelerating sales; cheap+grow (EV/EBIT 2.5x); cash 51% of mcap; cash &gt; EV (1.02x, net cash 51% mcap)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="18" customHeight="1"/>
-    <row r="45" ht="18" customHeight="1"/>
-    <row r="48">
-      <c r="A48" s="36" t="n"/>
-      <c r="B48" s="36" t="n"/>
-      <c r="C48" s="36" t="n"/>
-      <c r="D48" s="36" t="n"/>
-      <c r="E48" s="36" t="n"/>
-      <c r="F48" s="36" t="n"/>
-    </row>
-    <row r="49">
-      <c r="B49" s="26" t="inlineStr">
+          <t>·  Insider-aligned  (65% insider)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="16" customHeight="1">
+      <c r="B41" s="35" t="inlineStr">
+        <is>
+          <t>·  Cluster stack  (4 of 7 inflection signals)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="36" t="n"/>
+      <c r="B43" s="36" t="n"/>
+      <c r="C43" s="36" t="n"/>
+      <c r="D43" s="36" t="n"/>
+      <c r="E43" s="36" t="n"/>
+      <c r="F43" s="36" t="n"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="26" t="inlineStr">
         <is>
           <t>Asymmetry Workbook  ·  Sheet 46 of 50</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="16">
     <mergeCell ref="B40:E40"/>
     <mergeCell ref="B9:E9"/>
+    <mergeCell ref="B41:E41"/>
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="A20:E20"/>
     <mergeCell ref="B12:E12"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="B38:E38"/>
-    <mergeCell ref="A42:E42"/>
-    <mergeCell ref="B43:E45"/>
     <mergeCell ref="B7:E7"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A37:E37"/>
@@ -24049,7 +24033,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>20459466.81140074</v>
+        <v>20557711.54677471</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -24276,7 +24260,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>2.2538886</v>
+        <v>2.2647114</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -24435,7 +24419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -24449,7 +24433,7 @@
     <row r="1" ht="20" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>#48    1281.HK    LongiTech Smart Energy Holding Limited</t>
+          <t>#48    0725.HK    Perennial International Limited</t>
         </is>
       </c>
     </row>
@@ -24467,9 +24451,9 @@
           <t>Verdict</t>
         </is>
       </c>
-      <c r="C3" s="37" t="inlineStr">
-        <is>
-          <t>UNRESEARCHED</t>
+      <c r="C3" s="27" t="inlineStr">
+        <is>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="D3" s="26" t="inlineStr">
@@ -24478,7 +24462,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.016413963344826</v>
+        <v>1.019209861728622</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -24508,7 +24492,7 @@
       </c>
       <c r="B7" s="30" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
@@ -24520,7 +24504,7 @@
       </c>
       <c r="B8" s="30" t="inlineStr">
         <is>
-          <t>Independent Power and Renewable Electricity Producers</t>
+          <t>Electrical Equipment</t>
         </is>
       </c>
     </row>
@@ -24543,7 +24527,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>17239267.37836956</v>
+        <v>25007163.9423294</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -24553,7 +24537,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>19266963.3630279</v>
+        <v>50498298.96777866</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -24564,7 +24548,7 @@
       </c>
       <c r="B12" s="30" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>2025-12-31</t>
         </is>
       </c>
     </row>
@@ -24578,7 +24562,7 @@
     <row r="15" ht="22" customHeight="1">
       <c r="B15" s="32" t="inlineStr">
         <is>
-          <t>Unresearched. No qualitative thesis on file; ranking driven entirely by quantitative signals (see Score decomposition below).</t>
+          <t>Perennial International - electric cable family business; ~6% TTM dividend yield with intact payouts; P/B 0.46</t>
         </is>
       </c>
     </row>
@@ -24599,7 +24583,7 @@
         </is>
       </c>
       <c r="C21" s="22" t="n">
-        <v>0.6291497860677019</v>
+        <v>0.6381708462961632</v>
       </c>
       <c r="D21" s="33" t="inlineStr">
         <is>
@@ -24607,7 +24591,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.6629226316618847</v>
+        <v>0.4708091327139654</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -24617,7 +24601,7 @@
         </is>
       </c>
       <c r="C22" s="22" t="n">
-        <v>0.5145782893017455</v>
+        <v>0.5294406377810695</v>
       </c>
       <c r="D22" s="33" t="inlineStr">
         <is>
@@ -24625,7 +24609,7 @@
         </is>
       </c>
       <c r="E22" s="22" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
@@ -24643,7 +24627,7 @@
         </is>
       </c>
       <c r="E23" s="22" t="n">
-        <v>1</v>
+        <v>0.991</v>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
@@ -24653,7 +24637,7 @@
         </is>
       </c>
       <c r="C24" s="22" t="n">
-        <v>0.8794749681014746</v>
+        <v>0.820348</v>
       </c>
       <c r="D24" s="33" t="inlineStr">
         <is>
@@ -24661,7 +24645,7 @@
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>1.1434</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
@@ -24671,7 +24655,7 @@
         </is>
       </c>
       <c r="C25" s="22" t="n">
-        <v>0.4655292998699878</v>
+        <v>0.5524636352202518</v>
       </c>
       <c r="D25" s="33" t="inlineStr">
         <is>
@@ -24679,7 +24663,7 @@
         </is>
       </c>
       <c r="E25" s="34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
@@ -24696,17 +24680,15 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.13929923</v>
+        <v>0.41230643</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
           <t>NCAV / mcap (%)</t>
         </is>
       </c>
-      <c r="E28" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="E28" s="23" t="n">
+        <v>119.585308118896</v>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
@@ -24716,7 +24698,7 @@
         </is>
       </c>
       <c r="C29" s="22" t="n">
-        <v>-3.355922619636716</v>
+        <v>1.985515932474278</v>
       </c>
       <c r="D29" s="33" t="inlineStr">
         <is>
@@ -24724,7 +24706,7 @@
         </is>
       </c>
       <c r="E29" s="22" t="n">
-        <v>-7.396120066301267</v>
+        <v>-2.129477574667865</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
@@ -24744,7 +24726,7 @@
         </is>
       </c>
       <c r="E30" s="23" t="n">
-        <v>2.15667527759927</v>
+        <v>11.90882409257052</v>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
@@ -24754,7 +24736,7 @@
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>7.50352403384571</v>
+        <v>6.5666666</v>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
@@ -24762,7 +24744,7 @@
         </is>
       </c>
       <c r="E31" s="23" t="n">
-        <v>31.31714285714285</v>
+        <v>12.64845605700712</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
@@ -24772,7 +24754,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.8947578844443459</v>
+        <v>0.483827</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -24780,7 +24762,7 @@
         </is>
       </c>
       <c r="E32" s="23" t="n">
-        <v>65.373003</v>
+        <v>74.361</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
@@ -24789,10 +24771,8 @@
           <t>FCF yield (%)</t>
         </is>
       </c>
-      <c r="C33" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="C33" s="23" t="n">
+        <v>24.22527118078666</v>
       </c>
       <c r="D33" s="33" t="inlineStr">
         <is>
@@ -24812,7 +24792,7 @@
         </is>
       </c>
       <c r="C34" s="23" t="n">
-        <v>181.9727797636792</v>
+        <v>50.5420998322809</v>
       </c>
       <c r="D34" s="33" t="inlineStr">
         <is>
@@ -24820,7 +24800,7 @@
         </is>
       </c>
       <c r="E34" s="23" t="n">
-        <v>22.5586749656398</v>
+        <v>20.44019989165434</v>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
@@ -24830,7 +24810,7 @@
         </is>
       </c>
       <c r="C35" s="22" t="n">
-        <v>1.54376636882513</v>
+        <v>1.021921589561637</v>
       </c>
       <c r="D35" s="33" t="inlineStr">
         <is>
@@ -24838,7 +24818,7 @@
         </is>
       </c>
       <c r="E35" s="23" t="n">
-        <v>-24.14</v>
+        <v>32.5</v>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1">
@@ -24858,50 +24838,60 @@
     <row r="39" ht="16" customHeight="1">
       <c r="B39" s="35" t="inlineStr">
         <is>
-          <t>·  Sub-book  (P/B 0.14)</t>
+          <t>·  Sub-book  (P/B 0.41)</t>
         </is>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1">
       <c r="B40" s="35" t="inlineStr">
         <is>
-          <t>·  Insider-aligned  (65% insider)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="16" customHeight="1">
-      <c r="B41" s="35" t="inlineStr">
-        <is>
-          <t>·  Cluster stack  (4 of 7 inflection signals)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="36" t="n"/>
-      <c r="B43" s="36" t="n"/>
-      <c r="C43" s="36" t="n"/>
-      <c r="D43" s="36" t="n"/>
-      <c r="E43" s="36" t="n"/>
-      <c r="F43" s="36" t="n"/>
-    </row>
-    <row r="44">
-      <c r="B44" s="26" t="inlineStr">
+          <t>·  Insider-aligned  (74% insider)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>growth-flip; accelerating sales; cheap+grow (EV/EBIT 2.5x); cash 51% of mcap; cash &gt; EV (1.02x, net cash 51% mcap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1"/>
+    <row r="45" ht="18" customHeight="1"/>
+    <row r="48">
+      <c r="A48" s="36" t="n"/>
+      <c r="B48" s="36" t="n"/>
+      <c r="C48" s="36" t="n"/>
+      <c r="D48" s="36" t="n"/>
+      <c r="E48" s="36" t="n"/>
+      <c r="F48" s="36" t="n"/>
+    </row>
+    <row r="49">
+      <c r="B49" s="26" t="inlineStr">
         <is>
           <t>Asymmetry Workbook  ·  Sheet 48 of 50</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="17">
     <mergeCell ref="B40:E40"/>
     <mergeCell ref="B9:E9"/>
-    <mergeCell ref="B41:E41"/>
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="A20:E20"/>
     <mergeCell ref="B12:E12"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="B38:E38"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="B43:E45"/>
     <mergeCell ref="B7:E7"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A37:E37"/>
@@ -25027,7 +25017,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>29224919.38030916</v>
+        <v>29546465.8716598</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -25254,7 +25244,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.6022702</v>
+        <v>0.6088967</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -25987,7 +25977,7 @@
         </is>
       </c>
       <c r="C5" s="41" t="n">
-        <v>26385</v>
+        <v>26389</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>122</v>
@@ -25999,10 +25989,10 @@
         <v>99</v>
       </c>
       <c r="G5" s="31" t="n">
-        <v>25984</v>
+        <v>25988</v>
       </c>
       <c r="H5" s="42" t="n">
-        <v>1.519802918324806</v>
+        <v>1.519572549168214</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
@@ -26202,16 +26192,16 @@
         <v>2</v>
       </c>
       <c r="E16" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F16" s="34" t="n">
         <v>0</v>
       </c>
       <c r="G16" s="34" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H16" s="23" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17">
@@ -27533,7 +27523,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.214607294531874</v>
+        <v>1.213706119342358</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -27598,7 +27588,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>196398350.8262919</v>
+        <v>198008171.3658428</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -27662,7 +27652,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.671342612</v>
+        <v>0.67028805</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -27751,7 +27741,7 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.64328694</v>
+        <v>0.64855975</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
@@ -27771,7 +27761,7 @@
         </is>
       </c>
       <c r="C29" s="22" t="n">
-        <v>-1.47356998523237</v>
+        <v>-1.427733700674697</v>
       </c>
       <c r="D29" s="33" t="inlineStr">
         <is>
@@ -27807,7 +27797,7 @@
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>21.73689776387475</v>
+        <v>21.91506883475788</v>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
@@ -27825,7 +27815,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>1.06764828969794</v>
+        <v>1.076399494270387</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -27909,7 +27899,7 @@
     <row r="39" ht="16" customHeight="1">
       <c r="B39" s="35" t="inlineStr">
         <is>
-          <t>·  Sub-book  (P/B 0.64)</t>
+          <t>·  Sub-book  (P/B 0.65)</t>
         </is>
       </c>
     </row>
@@ -28080,7 +28070,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>129835458.4956091</v>
+        <v>129538583.7003687</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -28305,7 +28295,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.47688493</v>
+        <v>0.47579452</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Rebuild all books with the three new forensic archetypes + freshness gate
Regenerated the render-managed workbooks so arch_lifo_hidden_reserve,
arch_pension_overfunded, arch_dta_reversal and the tightened post_reorg
(freshness) firing sets are reflected.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/asymmetry_harvard_workbook.xlsx
+++ b/asymmetry_harvard_workbook.xlsx
@@ -15,8 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_2230_HK" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_3798_HK" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_4629_T" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_AWC_SI" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_003650_KS" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_003650_KS" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_AWC_SI" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_4301_T" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_IRC_BK" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_054800_KQ" sheetId="13" state="visible" r:id="rId13"/>
@@ -893,7 +893,7 @@
     <row r="1" ht="20" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>#07    003650.KS    Michang Oil Ind .Co.,Ltd.</t>
+          <t>#07    AWC.SI    Brook Crompton Holdings Ltd.</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.190631767830064</v>
+        <v>1.19387677304337</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -940,7 +940,7 @@
       </c>
       <c r="B6" s="30" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>SG</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="B7" s="30" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
@@ -964,7 +964,7 @@
       </c>
       <c r="B8" s="30" t="inlineStr">
         <is>
-          <t>Oil, Gas &amp; Consumable Fuels</t>
+          <t>Electrical Equipment</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
     </row>
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>129538583.7003727</v>
+        <v>15698515.16605616</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>265260383.0321121</v>
+        <v>47767733.03747177</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B12" s="30" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2025-12-31</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1022,7 @@
     <row r="15" ht="22" customHeight="1">
       <c r="B15" s="32" t="inlineStr">
         <is>
-          <t>Profitable Busan lubricants/white-oils maker (FY23 net income 47.6B KRW +104% YoY); 2.5% yield with only 6.6% payout signals net-cash hoard, classic Korean sub-book niche-leader setup</t>
+          <t>Brook Crompton - net-net + cash&gt;EV; Wolong as parent could squeeze out at low multiple = double-edged catalyst</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="C21" s="22" t="n">
-        <v>0.6220646644880169</v>
+        <v>0.6161324761871702</v>
       </c>
       <c r="D21" s="33" t="inlineStr">
         <is>
@@ -1051,7 +1051,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.7813682137134539</v>
+        <v>0.7365323562033702</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -1061,7 +1061,7 @@
         </is>
       </c>
       <c r="C22" s="22" t="n">
-        <v>0.4374380703008398</v>
+        <v>0.5018694881453837</v>
       </c>
       <c r="D22" s="33" t="inlineStr">
         <is>
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="C23" s="22" t="n">
-        <v>0.8846153846153845</v>
+        <v>0.7564102564102564</v>
       </c>
       <c r="D23" s="33" t="inlineStr">
         <is>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="C24" s="22" t="n">
-        <v>0.763853</v>
+        <v>0.81277</v>
       </c>
       <c r="D24" s="33" t="inlineStr">
         <is>
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>1.16</v>
+        <v>1.185</v>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
@@ -1115,7 +1115,7 @@
         </is>
       </c>
       <c r="C25" s="22" t="n">
-        <v>0.4460390065168427</v>
+        <v>0.578894638589458</v>
       </c>
       <c r="D25" s="33" t="inlineStr">
         <is>
@@ -1140,7 +1140,7 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.3814184820374598</v>
+        <v>0.4305136</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
         </is>
       </c>
       <c r="E28" s="23" t="n">
-        <v>195.4228046268257</v>
+        <v>186.2185523184757</v>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
@@ -1158,7 +1158,7 @@
         </is>
       </c>
       <c r="C29" s="22" t="n">
-        <v>0.502</v>
+        <v>1.614</v>
       </c>
       <c r="D29" s="33" t="inlineStr">
         <is>
@@ -1166,7 +1166,7 @@
         </is>
       </c>
       <c r="E29" s="22" t="n">
-        <v>-3.532483495983913</v>
+        <v>-13.95633802816901</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
@@ -1186,7 +1186,7 @@
         </is>
       </c>
       <c r="E30" s="23" t="n">
-        <v>48.19489607961939</v>
+        <v>13.92004707439961</v>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
@@ -1196,7 +1196,7 @@
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>3.257832481702135</v>
+        <v>8.142856999999999</v>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
@@ -1204,7 +1204,7 @@
         </is>
       </c>
       <c r="E31" s="23" t="n">
-        <v>12.06697403251717</v>
+        <v>2.30894308943089</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.47579452</v>
+        <v>0.3348663</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -1222,7 +1222,7 @@
         </is>
       </c>
       <c r="E32" s="23" t="n">
-        <v>50.244</v>
+        <v>66.086</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
@@ -1232,7 +1232,7 @@
         </is>
       </c>
       <c r="C33" s="23" t="n">
-        <v>3.22106752958146</v>
+        <v>4.09667276945568</v>
       </c>
       <c r="D33" s="33" t="inlineStr">
         <is>
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="C34" s="23" t="n">
-        <v>86.88917215306873</v>
+        <v>90.87835873445673</v>
       </c>
       <c r="D34" s="33" t="inlineStr">
         <is>
@@ -1260,7 +1260,7 @@
         </is>
       </c>
       <c r="E34" s="23" t="n">
-        <v>-6.109694716853889</v>
+        <v>-0.22712524334847</v>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
@@ -1270,7 +1270,7 @@
         </is>
       </c>
       <c r="C35" s="22" t="n">
-        <v>17.52230716826635</v>
+        <v>6.08519742575637</v>
       </c>
       <c r="D35" s="33" t="inlineStr">
         <is>
@@ -1278,7 +1278,7 @@
         </is>
       </c>
       <c r="E35" s="23" t="n">
-        <v>26.1</v>
+        <v>14.1</v>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1">
@@ -1305,14 +1305,14 @@
     <row r="40" ht="16" customHeight="1">
       <c r="B40" s="35" t="inlineStr">
         <is>
-          <t>·  Sub-book  (P/B 0.38)</t>
+          <t>·  Sub-book  (P/B 0.43)</t>
         </is>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1">
       <c r="B41" s="35" t="inlineStr">
         <is>
-          <t>·  Insider-aligned  (50% insider)</t>
+          <t>·  Insider-aligned  (66% insider)</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
     <row r="44" ht="18" customHeight="1">
       <c r="B44" s="12" t="inlineStr">
         <is>
-          <t>growth-flip; under-priced vs fundamentals; cheap+grow (EV/EBIT 0.1x); Graham net-net (mcap 0.51x NCAV); cash 150% of mcap; cash &gt; EV (17.52x, net cash 143% mcap)</t>
+          <t>growth-flip; accelerating sales; cheap+grow (EV/EBIT 1.0x); Graham net-net (mcap 0.54x NCAV); cash 108% of mcap; cash &gt; EV (6.09x, net cash 91% mcap)</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>185001225.2794647</v>
+        <v>185001225.2794639</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>425102384.579368</v>
+        <v>425102384.5793661</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -1985,7 +1985,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>78237641.18890381</v>
+        <v>78237641.18890361</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -1995,7 +1995,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>136153379.1378207</v>
+        <v>136153379.1378204</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -2173,10 +2173,8 @@
           <t>EV / EBIT</t>
         </is>
       </c>
-      <c r="C30" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="C30" s="22" t="n">
+        <v>0.4595209433628192</v>
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
@@ -2475,7 +2473,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>86400269.06174946</v>
+        <v>86400269.06174681</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -2485,7 +2483,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>621263383.7902402</v>
+        <v>621263383.7902211</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -3463,7 +3461,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>14694714.95424652</v>
+        <v>14694714.95424648</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -3473,7 +3471,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>8311024.856157303</v>
+        <v>8311024.856157282</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -3888,7 +3886,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.161336639699278</v>
+        <v>1.163897066936411</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -3951,7 +3949,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>97745653.94005205</v>
+        <v>97745653.94004904</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -3961,7 +3959,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>77102450.02260983</v>
+        <v>77102450.02260746</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -4069,7 +4067,7 @@
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>1.27</v>
+        <v>1.2728</v>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
@@ -4139,10 +4137,8 @@
           <t>EV / EBIT</t>
         </is>
       </c>
-      <c r="C30" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="C30" s="22" t="n">
+        <v>0.7374453048913777</v>
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
@@ -4441,7 +4437,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>69063217.17478943</v>
+        <v>69063217.17478731</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -4451,7 +4447,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>74515427.36626884</v>
+        <v>74515427.36626655</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -4935,7 +4931,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>98798555.87781906</v>
+        <v>98798555.87781604</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -4945,7 +4941,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>280815515.3520368</v>
+        <v>280815515.3520282</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -5123,10 +5119,8 @@
           <t>EV / EBIT</t>
         </is>
       </c>
-      <c r="C30" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="C30" s="22" t="n">
+        <v>1.926120339523525</v>
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
@@ -6059,7 +6053,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>36263429.07907248</v>
+        <v>36263429.07907232</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -6069,7 +6063,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>86615249.88943711</v>
+        <v>86615249.88943674</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -6555,7 +6549,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>18347168.83320999</v>
+        <v>18347168.83320943</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -6565,7 +6559,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>90551985.4721216</v>
+        <v>90551985.47211882</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -6743,10 +6737,8 @@
           <t>EV / EBIT</t>
         </is>
       </c>
-      <c r="C30" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="C30" s="22" t="n">
+        <v>0.9806606675872322</v>
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
@@ -7053,7 +7045,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>90146910.85052872</v>
+        <v>90146910.85052596</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -7063,7 +7055,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>85769277.6876678</v>
+        <v>85769277.68766516</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -7555,7 +7547,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>38413174.78646946</v>
+        <v>38413174.78646944</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -7565,7 +7557,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>184011076.5883501</v>
+        <v>184011076.58835</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -8041,7 +8033,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>48701579.34159088</v>
+        <v>48701579.34159086</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -8051,7 +8043,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>42302267.46344568</v>
+        <v>42302267.46344566</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -8231,10 +8223,8 @@
           <t>EV / EBIT</t>
         </is>
       </c>
-      <c r="C30" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="C30" s="22" t="n">
+        <v>-2.998632121052401</v>
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
@@ -8525,7 +8515,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>190876303.7740097</v>
+        <v>190876303.7740096</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -8535,7 +8525,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>169430939.0357057</v>
+        <v>169430939.0357056</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -8713,10 +8703,8 @@
           <t>EV / EBIT</t>
         </is>
       </c>
-      <c r="C30" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="C30" s="22" t="n">
+        <v>-4.937585342446557</v>
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
@@ -9023,7 +9011,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>24329555.49054528</v>
+        <v>24329555.49054453</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -9033,7 +9021,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>11671505.63693912</v>
+        <v>11671505.63693877</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -9211,10 +9199,8 @@
           <t>EV / EBIT</t>
         </is>
       </c>
-      <c r="C30" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="C30" s="22" t="n">
+        <v>1.742800322776044</v>
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
@@ -9517,7 +9503,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>331100479.5374721</v>
+        <v>331100479.537472</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -10005,7 +9991,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>21714424.70673323</v>
+        <v>21714424.70673309</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -10015,7 +10001,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>7273825.765494257</v>
+        <v>7273825.765494212</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -10497,7 +10483,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>37332395.3034389</v>
+        <v>37332395.30343874</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -10507,7 +10493,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>32923308.73264465</v>
+        <v>32923308.73264452</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -11080,7 +11066,7 @@
         </is>
       </c>
       <c r="H6" s="22" t="n">
-        <v>1.218387032001579</v>
+        <v>1.224320047113935</v>
       </c>
       <c r="I6" s="22" t="n">
         <v>0.5975976</v>
@@ -11184,22 +11170,22 @@
       </c>
       <c r="C9" s="17" t="inlineStr">
         <is>
-          <t>AWC.SI</t>
+          <t>003650.KS</t>
         </is>
       </c>
       <c r="D9" s="18" t="inlineStr">
         <is>
-          <t>Brook Crompton Holdings Ltd.</t>
+          <t>Michang Oil Ind .Co.,Ltd.</t>
         </is>
       </c>
       <c r="E9" s="19" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="F9" s="20" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="G9" s="21" t="inlineStr">
@@ -11208,16 +11194,16 @@
         </is>
       </c>
       <c r="H9" s="22" t="n">
-        <v>1.19387677304337</v>
+        <v>1.196379645329934</v>
       </c>
       <c r="I9" s="22" t="n">
-        <v>0.4305136</v>
+        <v>0.3814184820374598</v>
       </c>
       <c r="J9" s="23" t="n">
-        <v>3.28</v>
+        <v>2.77</v>
       </c>
       <c r="K9" s="22" t="n">
-        <v>0.3348663</v>
+        <v>0.47579452</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
@@ -11226,22 +11212,22 @@
       </c>
       <c r="C10" s="17" t="inlineStr">
         <is>
-          <t>003650.KS</t>
+          <t>AWC.SI</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
         <is>
-          <t>Michang Oil Ind .Co.,Ltd.</t>
+          <t>Brook Crompton Holdings Ltd.</t>
         </is>
       </c>
       <c r="E10" s="19" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="F10" s="20" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="G10" s="21" t="inlineStr">
@@ -11250,16 +11236,16 @@
         </is>
       </c>
       <c r="H10" s="22" t="n">
-        <v>1.190631767830064</v>
+        <v>1.19387677304337</v>
       </c>
       <c r="I10" s="22" t="n">
-        <v>0.3814184820374598</v>
+        <v>0.4305136</v>
       </c>
       <c r="J10" s="23" t="n">
-        <v>2.77</v>
+        <v>3.28</v>
       </c>
       <c r="K10" s="22" t="n">
-        <v>0.47579452</v>
+        <v>0.3348663</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
@@ -11502,7 +11488,7 @@
         </is>
       </c>
       <c r="H16" s="22" t="n">
-        <v>1.161336639699278</v>
+        <v>1.163897066936411</v>
       </c>
       <c r="I16" s="22" t="n">
         <v>0.9925171574056828</v>
@@ -13263,7 +13249,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>16725600.29102147</v>
+        <v>16725600.29102139</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -13273,7 +13259,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>55222673.83330967</v>
+        <v>55222673.83330944</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -13451,10 +13437,8 @@
           <t>EV / EBIT</t>
         </is>
       </c>
-      <c r="C30" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="C30" s="22" t="n">
+        <v>1.98262538471883</v>
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
@@ -13753,7 +13737,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>229039477.8522148</v>
+        <v>229039477.8522077</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -13763,7 +13747,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>291135327.5719234</v>
+        <v>291135327.5719145</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -14231,7 +14215,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>24004571.73281288</v>
+        <v>24004571.73281214</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -14241,7 +14225,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>41049810.50742675</v>
+        <v>41049810.50742549</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -14419,10 +14403,8 @@
           <t>EV / EBIT</t>
         </is>
       </c>
-      <c r="C30" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="C30" s="22" t="n">
+        <v>0.0915064559526798</v>
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
@@ -15225,7 +15207,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>58812410.08447552</v>
+        <v>58812410.08447371</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -15235,7 +15217,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>37014740.95624924</v>
+        <v>37014740.9562481</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -16211,7 +16193,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>88514613.8610754</v>
+        <v>88514613.86107269</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -16221,7 +16203,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>387812025.290559</v>
+        <v>387812025.2905471</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -16399,10 +16381,8 @@
           <t>EV / EBIT</t>
         </is>
       </c>
-      <c r="C30" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="C30" s="22" t="n">
+        <v>1.753430692904798</v>
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
@@ -16881,10 +16861,8 @@
           <t>EV / EBIT</t>
         </is>
       </c>
-      <c r="C30" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="C30" s="22" t="n">
+        <v>1.614595351131961</v>
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
@@ -17185,7 +17163,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>125759425.163269</v>
+        <v>125759425.1632687</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -17195,7 +17173,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>71113427.56021285</v>
+        <v>71113427.56021267</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -17669,7 +17647,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>50524003.6661768</v>
+        <v>50524003.66617677</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -17679,7 +17657,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>89795964.46359158</v>
+        <v>89795964.46359153</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -18167,7 +18145,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>34993764.18925142</v>
+        <v>34993764.18925035</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -18177,7 +18155,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>216015408.892177</v>
+        <v>216015408.8921704</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -18673,7 +18651,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>87952045.37611961</v>
+        <v>87952045.37611957</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -18683,7 +18661,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>461430088.9879614</v>
+        <v>461430088.9879612</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -19163,7 +19141,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>29658799.91638899</v>
+        <v>29658799.91638808</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -19173,7 +19151,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>89068535.34864391</v>
+        <v>89068535.34864119</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -19653,7 +19631,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>64845983.34468651</v>
+        <v>64845983.34468452</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -19663,7 +19641,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>390351789.1708</v>
+        <v>390351789.170788</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -20627,7 +20605,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>64179093.31776381</v>
+        <v>64179093.31776353</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -20637,7 +20615,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>82321438.99549031</v>
+        <v>82321438.99548995</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -21123,7 +21101,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>20557711.54677534</v>
+        <v>20557711.54677471</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -21133,7 +21111,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>8563148.622397322</v>
+        <v>8563148.62239706</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -21617,7 +21595,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>25007163.94232941</v>
+        <v>25007163.9423294</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -21627,7 +21605,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>50498298.96777868</v>
+        <v>50498298.96777866</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -22107,7 +22085,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>29546465.87166071</v>
+        <v>29546465.8716598</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -22117,7 +22095,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>43532230.22913835</v>
+        <v>43532230.22913702</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -22601,7 +22579,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>80246742.39991665</v>
+        <v>80246742.39991631</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -22611,7 +22589,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>145366592.7187284</v>
+        <v>145366592.7187277</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -23097,7 +23075,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>134233026.9123783</v>
+        <v>134233026.9123742</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -23107,7 +23085,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>275616874.9640363</v>
+        <v>275616874.9640279</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -23589,7 +23567,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>96779704.39331056</v>
+        <v>96779704.39330758</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -23599,7 +23577,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>293732750.4359149</v>
+        <v>293732750.4359059</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -24073,7 +24051,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>60319815.14114141</v>
+        <v>60319815.14114115</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -24083,7 +24061,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>147863210.4322873</v>
+        <v>147863210.4322867</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -24563,7 +24541,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>45157985.92321968</v>
+        <v>45157985.92321829</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -24573,7 +24551,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>201923506.9211402</v>
+        <v>201923506.921134</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -25057,7 +25035,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>268537192.4160213</v>
+        <v>268537192.4160212</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -25067,7 +25045,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>735679467.6824063</v>
+        <v>735679467.6824059</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -26559,7 +26537,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.218387032001579</v>
+        <v>1.224320047113935</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -26624,7 +26602,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>50583538.93268108</v>
+        <v>50583538.93268106</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -26634,7 +26612,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>82663114.82569575</v>
+        <v>82663114.82569572</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -26742,7 +26720,7 @@
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>1.15</v>
+        <v>1.1556</v>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
@@ -26812,10 +26790,8 @@
           <t>EV / EBIT</t>
         </is>
       </c>
-      <c r="C30" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="C30" s="22" t="n">
+        <v>1.244281797914842</v>
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
@@ -27134,7 +27110,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>183954166.1063844</v>
+        <v>183954166.1063843</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -27314,10 +27290,8 @@
           <t>EV / EBIT</t>
         </is>
       </c>
-      <c r="C30" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="C30" s="22" t="n">
+        <v>0.9912811803599012</v>
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
@@ -27608,7 +27582,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>71024071.39044285</v>
+        <v>71024071.39044254</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -27618,7 +27592,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>216405193.725382</v>
+        <v>216405193.725381</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -28014,7 +27988,7 @@
     <row r="1" ht="20" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>#06    AWC.SI    Brook Crompton Holdings Ltd.</t>
+          <t>#06    003650.KS    Michang Oil Ind .Co.,Ltd.</t>
         </is>
       </c>
     </row>
@@ -28043,7 +28017,7 @@
         </is>
       </c>
       <c r="E3" s="28" t="n">
-        <v>1.19387677304337</v>
+        <v>1.196379645329934</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -28061,7 +28035,7 @@
       </c>
       <c r="B6" s="30" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>KR</t>
         </is>
       </c>
     </row>
@@ -28073,7 +28047,7 @@
       </c>
       <c r="B7" s="30" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
     </row>
@@ -28085,7 +28059,7 @@
       </c>
       <c r="B8" s="30" t="inlineStr">
         <is>
-          <t>Electrical Equipment</t>
+          <t>Oil, Gas &amp; Consumable Fuels</t>
         </is>
       </c>
     </row>
@@ -28097,7 +28071,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Nano Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
     </row>
@@ -28108,7 +28082,7 @@
         </is>
       </c>
       <c r="B10" s="31" t="n">
-        <v>15698515.16605616</v>
+        <v>129538583.7003687</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -28118,7 +28092,7 @@
         </is>
       </c>
       <c r="B11" s="31" t="n">
-        <v>47767733.03747177</v>
+        <v>265260383.032104</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -28129,7 +28103,7 @@
       </c>
       <c r="B12" s="30" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-03-31</t>
         </is>
       </c>
     </row>
@@ -28143,7 +28117,7 @@
     <row r="15" ht="22" customHeight="1">
       <c r="B15" s="32" t="inlineStr">
         <is>
-          <t>Brook Crompton - net-net + cash&gt;EV; Wolong as parent could squeeze out at low multiple = double-edged catalyst</t>
+          <t>Profitable Busan lubricants/white-oils maker (FY23 net income 47.6B KRW +104% YoY); 2.5% yield with only 6.6% payout signals net-cash hoard, classic Korean sub-book niche-leader setup</t>
         </is>
       </c>
     </row>
@@ -28164,7 +28138,7 @@
         </is>
       </c>
       <c r="C21" s="22" t="n">
-        <v>0.6161324761871702</v>
+        <v>0.6220646644880169</v>
       </c>
       <c r="D21" s="33" t="inlineStr">
         <is>
@@ -28172,7 +28146,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>0.7365323562033702</v>
+        <v>0.7813682137134539</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -28182,7 +28156,7 @@
         </is>
       </c>
       <c r="C22" s="22" t="n">
-        <v>0.5018694881453837</v>
+        <v>0.4374380703008398</v>
       </c>
       <c r="D22" s="33" t="inlineStr">
         <is>
@@ -28200,7 +28174,7 @@
         </is>
       </c>
       <c r="C23" s="22" t="n">
-        <v>0.7564102564102564</v>
+        <v>0.8846153846153845</v>
       </c>
       <c r="D23" s="33" t="inlineStr">
         <is>
@@ -28218,7 +28192,7 @@
         </is>
       </c>
       <c r="C24" s="22" t="n">
-        <v>0.81277</v>
+        <v>0.763853</v>
       </c>
       <c r="D24" s="33" t="inlineStr">
         <is>
@@ -28226,7 +28200,7 @@
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>1.185</v>
+        <v>1.1656</v>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
@@ -28236,7 +28210,7 @@
         </is>
       </c>
       <c r="C25" s="22" t="n">
-        <v>0.578894638589458</v>
+        <v>0.4460390065168427</v>
       </c>
       <c r="D25" s="33" t="inlineStr">
         <is>
@@ -28261,7 +28235,7 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>0.4305136</v>
+        <v>0.3814184820374598</v>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
@@ -28269,7 +28243,7 @@
         </is>
       </c>
       <c r="E28" s="23" t="n">
-        <v>186.2185523184757</v>
+        <v>195.4228046268257</v>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
@@ -28279,7 +28253,7 @@
         </is>
       </c>
       <c r="C29" s="22" t="n">
-        <v>1.614</v>
+        <v>0.502</v>
       </c>
       <c r="D29" s="33" t="inlineStr">
         <is>
@@ -28287,7 +28261,7 @@
         </is>
       </c>
       <c r="E29" s="22" t="n">
-        <v>-13.95633802816901</v>
+        <v>-3.532483495983913</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
@@ -28296,10 +28270,8 @@
           <t>EV / EBIT</t>
         </is>
       </c>
-      <c r="C30" s="25" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="C30" s="22" t="n">
+        <v>0.5830299613427031</v>
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
@@ -28307,7 +28279,7 @@
         </is>
       </c>
       <c r="E30" s="23" t="n">
-        <v>13.92004707439961</v>
+        <v>48.19489607961939</v>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
@@ -28317,7 +28289,7 @@
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>8.142856999999999</v>
+        <v>3.257832481702135</v>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
@@ -28325,7 +28297,7 @@
         </is>
       </c>
       <c r="E31" s="23" t="n">
-        <v>2.30894308943089</v>
+        <v>12.06697403251717</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
@@ -28335,7 +28307,7 @@
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>0.3348663</v>
+        <v>0.47579452</v>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
@@ -28343,7 +28315,7 @@
         </is>
       </c>
       <c r="E32" s="23" t="n">
-        <v>66.086</v>
+        <v>50.244</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
@@ -28353,7 +28325,7 @@
         </is>
       </c>
       <c r="C33" s="23" t="n">
-        <v>4.09667276945568</v>
+        <v>3.22106752958146</v>
       </c>
       <c r="D33" s="33" t="inlineStr">
         <is>
@@ -28373,7 +28345,7 @@
         </is>
       </c>
       <c r="C34" s="23" t="n">
-        <v>90.87835873445673</v>
+        <v>86.88917215306873</v>
       </c>
       <c r="D34" s="33" t="inlineStr">
         <is>
@@ -28381,7 +28353,7 @@
         </is>
       </c>
       <c r="E34" s="23" t="n">
-        <v>-0.22712524334847</v>
+        <v>-6.109694716853889</v>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
@@ -28391,7 +28363,7 @@
         </is>
       </c>
       <c r="C35" s="22" t="n">
-        <v>6.08519742575637</v>
+        <v>17.52230716826635</v>
       </c>
       <c r="D35" s="33" t="inlineStr">
         <is>
@@ -28399,7 +28371,7 @@
         </is>
       </c>
       <c r="E35" s="23" t="n">
-        <v>14.1</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1">
@@ -28426,14 +28398,14 @@
     <row r="40" ht="16" customHeight="1">
       <c r="B40" s="35" t="inlineStr">
         <is>
-          <t>·  Sub-book  (P/B 0.43)</t>
+          <t>·  Sub-book  (P/B 0.38)</t>
         </is>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1">
       <c r="B41" s="35" t="inlineStr">
         <is>
-          <t>·  Insider-aligned  (66% insider)</t>
+          <t>·  Insider-aligned  (50% insider)</t>
         </is>
       </c>
     </row>
@@ -28447,7 +28419,7 @@
     <row r="44" ht="18" customHeight="1">
       <c r="B44" s="12" t="inlineStr">
         <is>
-          <t>growth-flip; accelerating sales; cheap+grow (EV/EBIT 1.0x); Graham net-net (mcap 0.54x NCAV); cash 108% of mcap; cash &gt; EV (6.09x, net cash 91% mcap)</t>
+          <t>growth-flip; under-priced vs fundamentals; cheap+grow (EV/EBIT 0.1x); Graham net-net (mcap 0.51x NCAV); cash 150% of mcap; cash &gt; EV (17.52x, net cash 143% mcap)</t>
         </is>
       </c>
     </row>

</xml_diff>